<commit_message>
Big update: Aztec art (procedural), animations, particles, sound, buy menu; Super/Gods bonus modes; bug fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011QYnJU3qzdAzbD5jkFKhoX
</commit_message>
<xml_diff>
--- a/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
+++ b/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
@@ -11,13 +11,15 @@
     <sheet name="bonushunt" sheetId="2" r:id="rId2"/>
     <sheet name="jaguar" sheetId="3" r:id="rId3"/>
     <sheet name="bonus" sheetId="4" r:id="rId4"/>
+    <sheet name="superbonus" sheetId="5" r:id="rId5"/>
+    <sheet name="godbonus" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="108">
   <si>
     <t>Win Ranges</t>
   </si>
@@ -290,6 +292,57 @@
   </si>
   <si>
     <t>8948.719805485023</t>
+  </si>
+  <si>
+    <t>19200.00000150739</t>
+  </si>
+  <si>
+    <t>49.219989158790916</t>
+  </si>
+  <si>
+    <t>18694.101466905176</t>
+  </si>
+  <si>
+    <t>72.04819929392171</t>
+  </si>
+  <si>
+    <t>20202.45683450384</t>
+  </si>
+  <si>
+    <t>181.71508609230705</t>
+  </si>
+  <si>
+    <t>18872.22849952668</t>
+  </si>
+  <si>
+    <t>28800.00000114848</t>
+  </si>
+  <si>
+    <t>49.16263194675667</t>
+  </si>
+  <si>
+    <t>2034</t>
+  </si>
+  <si>
+    <t>28925.64882408997</t>
+  </si>
+  <si>
+    <t>72.01293114912663</t>
+  </si>
+  <si>
+    <t>1388</t>
+  </si>
+  <si>
+    <t>29385.738842274877</t>
+  </si>
+  <si>
+    <t>181.54103514946814</t>
+  </si>
+  <si>
+    <t>550</t>
+  </si>
+  <si>
+    <t>28267.391331219074</t>
   </si>
 </sst>
 </file>
@@ -3957,4 +4010,1674 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P43"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>154.505</v>
+      </c>
+      <c r="C3">
+        <v>1.551405472234485E-05</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>155.277</v>
+      </c>
+      <c r="C4">
+        <v>4.311858053858259E-05</v>
+      </c>
+      <c r="F4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K4">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>48.413</v>
+      </c>
+      <c r="C5">
+        <v>0.0003463252266073023</v>
+      </c>
+      <c r="F5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" t="s">
+        <v>6</v>
+      </c>
+      <c r="K5">
+        <v>2432</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>27.679</v>
+      </c>
+      <c r="C6">
+        <v>0.001329718400825744</v>
+      </c>
+      <c r="F6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K6">
+        <v>4097</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>13.313</v>
+      </c>
+      <c r="C7">
+        <v>0.005544504689862224</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7">
+        <v>8216</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>5.093</v>
+      </c>
+      <c r="C8">
+        <v>0.03326561542230876</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="J8" t="s">
+        <v>9</v>
+      </c>
+      <c r="K8">
+        <v>20544</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>4.825</v>
+      </c>
+      <c r="C9">
+        <v>0.07490878573742843</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" t="s">
+        <v>10</v>
+      </c>
+      <c r="K9">
+        <v>20767</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10">
+        <v>5.219</v>
+      </c>
+      <c r="C10">
+        <v>0.1366294583021566</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="J10" t="s">
+        <v>11</v>
+      </c>
+      <c r="K10">
+        <v>18476</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>11.234</v>
+      </c>
+      <c r="C11">
+        <v>0.1088880388687363</v>
+      </c>
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="J11" t="s">
+        <v>12</v>
+      </c>
+      <c r="K11">
+        <v>8319</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12">
+        <v>12.027</v>
+      </c>
+      <c r="C12">
+        <v>0.1594956864616534</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J12" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12">
+        <v>7576</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13">
+        <v>15.913</v>
+      </c>
+      <c r="C13">
+        <v>0.2169138578186219</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13">
+        <v>5540</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14">
+        <v>52.39</v>
+      </c>
+      <c r="C14">
+        <v>0.1280334090932304</v>
+      </c>
+      <c r="F14" t="s">
+        <v>15</v>
+      </c>
+      <c r="J14" t="s">
+        <v>15</v>
+      </c>
+      <c r="K14">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15">
+        <v>292.987</v>
+      </c>
+      <c r="C15">
+        <v>0.04129767627518412</v>
+      </c>
+      <c r="F15" t="s">
+        <v>16</v>
+      </c>
+      <c r="J15" t="s">
+        <v>16</v>
+      </c>
+      <c r="K15">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16">
+        <v>511.771</v>
+      </c>
+      <c r="C16">
+        <v>0.03549886770219404</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>17</v>
+      </c>
+      <c r="K16">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17">
+        <v>2117.195</v>
+      </c>
+      <c r="C17">
+        <v>0.01532874738603764</v>
+      </c>
+      <c r="F17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K17">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18">
+        <v>22817.264</v>
+      </c>
+      <c r="C18">
+        <v>0.002191334274341069</v>
+      </c>
+      <c r="F18" t="s">
+        <v>20</v>
+      </c>
+      <c r="J18" t="s">
+        <v>20</v>
+      </c>
+      <c r="K18">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" t="s">
+        <v>34</v>
+      </c>
+      <c r="M22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16">
+      <c r="B23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" t="s">
+        <v>33</v>
+      </c>
+      <c r="H23" t="s">
+        <v>31</v>
+      </c>
+      <c r="I23" t="s">
+        <v>32</v>
+      </c>
+      <c r="J23" t="s">
+        <v>33</v>
+      </c>
+      <c r="N23" t="s">
+        <v>31</v>
+      </c>
+      <c r="O23" t="s">
+        <v>32</v>
+      </c>
+      <c r="P23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24">
+        <v>329.38</v>
+      </c>
+      <c r="C24">
+        <v>52.65</v>
+      </c>
+      <c r="D24">
+        <v>6.45</v>
+      </c>
+      <c r="G24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24">
+        <v>304</v>
+      </c>
+      <c r="I24">
+        <v>1896</v>
+      </c>
+      <c r="J24">
+        <v>15503</v>
+      </c>
+      <c r="M24" t="s">
+        <v>22</v>
+      </c>
+      <c r="N24">
+        <v>20962.1</v>
+      </c>
+      <c r="O24">
+        <v>19800.4</v>
+      </c>
+      <c r="P24">
+        <v>18932.3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25">
+        <v>223.96</v>
+      </c>
+      <c r="C25">
+        <v>31.15</v>
+      </c>
+      <c r="D25">
+        <v>4.35</v>
+      </c>
+      <c r="G25" t="s">
+        <v>23</v>
+      </c>
+      <c r="H25">
+        <v>447</v>
+      </c>
+      <c r="I25">
+        <v>3210</v>
+      </c>
+      <c r="J25">
+        <v>22990</v>
+      </c>
+      <c r="M25" t="s">
+        <v>23</v>
+      </c>
+      <c r="N25">
+        <v>19000.5</v>
+      </c>
+      <c r="O25">
+        <v>19689.6</v>
+      </c>
+      <c r="P25">
+        <v>19184.9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>213.3</v>
+      </c>
+      <c r="C26">
+        <v>30.48</v>
+      </c>
+      <c r="D26">
+        <v>4.48</v>
+      </c>
+      <c r="G26" t="s">
+        <v>24</v>
+      </c>
+      <c r="H26">
+        <v>467</v>
+      </c>
+      <c r="I26">
+        <v>3285</v>
+      </c>
+      <c r="J26">
+        <v>22324</v>
+      </c>
+      <c r="M26" t="s">
+        <v>24</v>
+      </c>
+      <c r="N26">
+        <v>17820.4</v>
+      </c>
+      <c r="O26">
+        <v>19570.9</v>
+      </c>
+      <c r="P26">
+        <v>19657.3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27">
+        <v>113.04</v>
+      </c>
+      <c r="C27">
+        <v>17.54</v>
+      </c>
+      <c r="D27">
+        <v>2.79</v>
+      </c>
+      <c r="G27" t="s">
+        <v>25</v>
+      </c>
+      <c r="H27">
+        <v>883</v>
+      </c>
+      <c r="I27">
+        <v>5695</v>
+      </c>
+      <c r="J27">
+        <v>35820</v>
+      </c>
+      <c r="M27" t="s">
+        <v>25</v>
+      </c>
+      <c r="N27">
+        <v>20416.3</v>
+      </c>
+      <c r="O27">
+        <v>19195.6</v>
+      </c>
+      <c r="P27">
+        <v>19131.8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16">
+      <c r="A28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28">
+        <v>61.44</v>
+      </c>
+      <c r="C28">
+        <v>12.52</v>
+      </c>
+      <c r="D28">
+        <v>2.3</v>
+      </c>
+      <c r="G28" t="s">
+        <v>26</v>
+      </c>
+      <c r="H28">
+        <v>1638</v>
+      </c>
+      <c r="I28">
+        <v>7988</v>
+      </c>
+      <c r="J28">
+        <v>43510</v>
+      </c>
+      <c r="M28" t="s">
+        <v>26</v>
+      </c>
+      <c r="N28">
+        <v>18128.3</v>
+      </c>
+      <c r="O28">
+        <v>18886.2</v>
+      </c>
+      <c r="P28">
+        <v>19122.8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29">
+        <v>45.55</v>
+      </c>
+      <c r="C29">
+        <v>9.57</v>
+      </c>
+      <c r="D29">
+        <v>2.14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29">
+        <v>2196</v>
+      </c>
+      <c r="I29">
+        <v>10451</v>
+      </c>
+      <c r="J29">
+        <v>46789</v>
+      </c>
+      <c r="M29" t="s">
+        <v>27</v>
+      </c>
+      <c r="N29">
+        <v>20312.2</v>
+      </c>
+      <c r="O29">
+        <v>19032.1</v>
+      </c>
+      <c r="P29">
+        <v>19112.2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30">
+        <v>34.73</v>
+      </c>
+      <c r="C30">
+        <v>8.460000000000001</v>
+      </c>
+      <c r="D30">
+        <v>2</v>
+      </c>
+      <c r="G30" t="s">
+        <v>28</v>
+      </c>
+      <c r="H30">
+        <v>2877</v>
+      </c>
+      <c r="I30">
+        <v>11822</v>
+      </c>
+      <c r="J30">
+        <v>49984</v>
+      </c>
+      <c r="M30" t="s">
+        <v>28</v>
+      </c>
+      <c r="N30">
+        <v>18675.1</v>
+      </c>
+      <c r="O30">
+        <v>19226.3</v>
+      </c>
+      <c r="P30">
+        <v>19360.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31">
+        <v>23.91</v>
+      </c>
+      <c r="C31">
+        <v>5.62</v>
+      </c>
+      <c r="D31">
+        <v>1.54</v>
+      </c>
+      <c r="G31" t="s">
+        <v>29</v>
+      </c>
+      <c r="H31">
+        <v>4177</v>
+      </c>
+      <c r="I31">
+        <v>17776</v>
+      </c>
+      <c r="J31">
+        <v>64923</v>
+      </c>
+      <c r="M31" t="s">
+        <v>29</v>
+      </c>
+      <c r="N31">
+        <v>19729.6</v>
+      </c>
+      <c r="O31">
+        <v>19608.5</v>
+      </c>
+      <c r="P31">
+        <v>19066.2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32">
+        <v>21.48</v>
+      </c>
+      <c r="C32">
+        <v>5.49</v>
+      </c>
+      <c r="D32">
+        <v>1.5</v>
+      </c>
+      <c r="G32" t="s">
+        <v>30</v>
+      </c>
+      <c r="H32">
+        <v>4665</v>
+      </c>
+      <c r="I32">
+        <v>18248</v>
+      </c>
+      <c r="J32">
+        <v>66734</v>
+      </c>
+      <c r="M32" t="s">
+        <v>30</v>
+      </c>
+      <c r="N32">
+        <v>18951.7</v>
+      </c>
+      <c r="O32">
+        <v>19042.7</v>
+      </c>
+      <c r="P32">
+        <v>19254.3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="B38" t="s">
+        <v>37</v>
+      </c>
+      <c r="C38" t="s">
+        <v>38</v>
+      </c>
+      <c r="D38" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" t="s">
+        <v>79</v>
+      </c>
+      <c r="C39" t="s">
+        <v>80</v>
+      </c>
+      <c r="D39" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40" t="s">
+        <v>92</v>
+      </c>
+      <c r="C40" t="s">
+        <v>83</v>
+      </c>
+      <c r="D40" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41" t="s">
+        <v>94</v>
+      </c>
+      <c r="C41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D41" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" t="s">
+        <v>96</v>
+      </c>
+      <c r="C42" t="s">
+        <v>89</v>
+      </c>
+      <c r="D42" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" t="s">
+        <v>57</v>
+      </c>
+      <c r="D43" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P43"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>101.95</v>
+      </c>
+      <c r="C3">
+        <v>1.567845452555597E-05</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>158.118</v>
+      </c>
+      <c r="C4">
+        <v>2.84908054347311E-05</v>
+      </c>
+      <c r="F4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K4">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>73.916</v>
+      </c>
+      <c r="C5">
+        <v>0.0001490274905700036</v>
+      </c>
+      <c r="F5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" t="s">
+        <v>6</v>
+      </c>
+      <c r="K5">
+        <v>1355</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>49.631</v>
+      </c>
+      <c r="C6">
+        <v>0.0004848806888288293</v>
+      </c>
+      <c r="F6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K6">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>24.192</v>
+      </c>
+      <c r="C7">
+        <v>0.001992863410510948</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7">
+        <v>4132</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>8.17</v>
+      </c>
+      <c r="C8">
+        <v>0.01390013261520781</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="J8" t="s">
+        <v>9</v>
+      </c>
+      <c r="K8">
+        <v>12220</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>6.066</v>
+      </c>
+      <c r="C9">
+        <v>0.0400348416289838</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" t="s">
+        <v>10</v>
+      </c>
+      <c r="K9">
+        <v>16438</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10">
+        <v>4.665</v>
+      </c>
+      <c r="C10">
+        <v>0.1031304321006027</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="J10" t="s">
+        <v>11</v>
+      </c>
+      <c r="K10">
+        <v>21353</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>8.234</v>
+      </c>
+      <c r="C11">
+        <v>0.09933730499787798</v>
+      </c>
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="J11" t="s">
+        <v>12</v>
+      </c>
+      <c r="K11">
+        <v>12089</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12">
+        <v>7.647</v>
+      </c>
+      <c r="C12">
+        <v>0.1680561171908286</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J12" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12">
+        <v>13007</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13">
+        <v>9.409000000000001</v>
+      </c>
+      <c r="C13">
+        <v>0.2445108232349976</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13">
+        <v>10562</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14">
+        <v>26.686</v>
+      </c>
+      <c r="C14">
+        <v>0.1680956891126261</v>
+      </c>
+      <c r="F14" t="s">
+        <v>15</v>
+      </c>
+      <c r="J14" t="s">
+        <v>15</v>
+      </c>
+      <c r="K14">
+        <v>3916</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15">
+        <v>149.584</v>
+      </c>
+      <c r="C15">
+        <v>0.05351409748226453</v>
+      </c>
+      <c r="F15" t="s">
+        <v>16</v>
+      </c>
+      <c r="J15" t="s">
+        <v>16</v>
+      </c>
+      <c r="K15">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16">
+        <v>284.317</v>
+      </c>
+      <c r="C16">
+        <v>0.04251228596928779</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>17</v>
+      </c>
+      <c r="K16">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17">
+        <v>974.333</v>
+      </c>
+      <c r="C17">
+        <v>0.0220922933156408</v>
+      </c>
+      <c r="F17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K17">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18">
+        <v>17975.124</v>
+      </c>
+      <c r="C18">
+        <v>0.001854434014131015</v>
+      </c>
+      <c r="F18" t="s">
+        <v>20</v>
+      </c>
+      <c r="J18" t="s">
+        <v>20</v>
+      </c>
+      <c r="K18">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" t="s">
+        <v>34</v>
+      </c>
+      <c r="M22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16">
+      <c r="B23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" t="s">
+        <v>33</v>
+      </c>
+      <c r="H23" t="s">
+        <v>31</v>
+      </c>
+      <c r="I23" t="s">
+        <v>32</v>
+      </c>
+      <c r="J23" t="s">
+        <v>33</v>
+      </c>
+      <c r="N23" t="s">
+        <v>31</v>
+      </c>
+      <c r="O23" t="s">
+        <v>32</v>
+      </c>
+      <c r="P23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24">
+        <v>344.69</v>
+      </c>
+      <c r="C24">
+        <v>58.37</v>
+      </c>
+      <c r="D24">
+        <v>7.07</v>
+      </c>
+      <c r="G24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24">
+        <v>290</v>
+      </c>
+      <c r="I24">
+        <v>1712</v>
+      </c>
+      <c r="J24">
+        <v>14150</v>
+      </c>
+      <c r="M24" t="s">
+        <v>22</v>
+      </c>
+      <c r="N24">
+        <v>34350.3</v>
+      </c>
+      <c r="O24">
+        <v>29595.1</v>
+      </c>
+      <c r="P24">
+        <v>28442.4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25">
+        <v>251.49</v>
+      </c>
+      <c r="C25">
+        <v>34.52</v>
+      </c>
+      <c r="D25">
+        <v>4.71</v>
+      </c>
+      <c r="G25" t="s">
+        <v>23</v>
+      </c>
+      <c r="H25">
+        <v>398</v>
+      </c>
+      <c r="I25">
+        <v>2901</v>
+      </c>
+      <c r="J25">
+        <v>21255</v>
+      </c>
+      <c r="M25" t="s">
+        <v>23</v>
+      </c>
+      <c r="N25">
+        <v>27068.9</v>
+      </c>
+      <c r="O25">
+        <v>28671.5</v>
+      </c>
+      <c r="P25">
+        <v>28773.9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>230.17</v>
+      </c>
+      <c r="C26">
+        <v>33.37</v>
+      </c>
+      <c r="D26">
+        <v>4.85</v>
+      </c>
+      <c r="G26" t="s">
+        <v>24</v>
+      </c>
+      <c r="H26">
+        <v>434</v>
+      </c>
+      <c r="I26">
+        <v>2998</v>
+      </c>
+      <c r="J26">
+        <v>20612</v>
+      </c>
+      <c r="M26" t="s">
+        <v>24</v>
+      </c>
+      <c r="N26">
+        <v>28062.7</v>
+      </c>
+      <c r="O26">
+        <v>28794.2</v>
+      </c>
+      <c r="P26">
+        <v>29002.8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27">
+        <v>122.66</v>
+      </c>
+      <c r="C27">
+        <v>19.31</v>
+      </c>
+      <c r="D27">
+        <v>2.98</v>
+      </c>
+      <c r="G27" t="s">
+        <v>25</v>
+      </c>
+      <c r="H27">
+        <v>815</v>
+      </c>
+      <c r="I27">
+        <v>5181</v>
+      </c>
+      <c r="J27">
+        <v>33505</v>
+      </c>
+      <c r="M27" t="s">
+        <v>25</v>
+      </c>
+      <c r="N27">
+        <v>28304.2</v>
+      </c>
+      <c r="O27">
+        <v>28514</v>
+      </c>
+      <c r="P27">
+        <v>28775.7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16">
+      <c r="A28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28">
+        <v>66.29000000000001</v>
+      </c>
+      <c r="C28">
+        <v>13.52</v>
+      </c>
+      <c r="D28">
+        <v>2.44</v>
+      </c>
+      <c r="G28" t="s">
+        <v>26</v>
+      </c>
+      <c r="H28">
+        <v>1514</v>
+      </c>
+      <c r="I28">
+        <v>7392</v>
+      </c>
+      <c r="J28">
+        <v>40910</v>
+      </c>
+      <c r="M28" t="s">
+        <v>26</v>
+      </c>
+      <c r="N28">
+        <v>26635.1</v>
+      </c>
+      <c r="O28">
+        <v>28789.6</v>
+      </c>
+      <c r="P28">
+        <v>28586.1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29">
+        <v>50.17</v>
+      </c>
+      <c r="C29">
+        <v>10.45</v>
+      </c>
+      <c r="D29">
+        <v>2.28</v>
+      </c>
+      <c r="G29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29">
+        <v>1994</v>
+      </c>
+      <c r="I29">
+        <v>9568</v>
+      </c>
+      <c r="J29">
+        <v>43887</v>
+      </c>
+      <c r="M29" t="s">
+        <v>27</v>
+      </c>
+      <c r="N29">
+        <v>29093</v>
+      </c>
+      <c r="O29">
+        <v>28505.5</v>
+      </c>
+      <c r="P29">
+        <v>28609.3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30">
+        <v>37.81</v>
+      </c>
+      <c r="C30">
+        <v>9.16</v>
+      </c>
+      <c r="D30">
+        <v>2.13</v>
+      </c>
+      <c r="G30" t="s">
+        <v>28</v>
+      </c>
+      <c r="H30">
+        <v>2642</v>
+      </c>
+      <c r="I30">
+        <v>10919</v>
+      </c>
+      <c r="J30">
+        <v>46970</v>
+      </c>
+      <c r="M30" t="s">
+        <v>28</v>
+      </c>
+      <c r="N30">
+        <v>27522.1</v>
+      </c>
+      <c r="O30">
+        <v>28662.8</v>
+      </c>
+      <c r="P30">
+        <v>28912.3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31">
+        <v>26.23</v>
+      </c>
+      <c r="C31">
+        <v>6.15</v>
+      </c>
+      <c r="D31">
+        <v>1.62</v>
+      </c>
+      <c r="G31" t="s">
+        <v>29</v>
+      </c>
+      <c r="H31">
+        <v>3813</v>
+      </c>
+      <c r="I31">
+        <v>16262</v>
+      </c>
+      <c r="J31">
+        <v>61789</v>
+      </c>
+      <c r="M31" t="s">
+        <v>29</v>
+      </c>
+      <c r="N31">
+        <v>29117.8</v>
+      </c>
+      <c r="O31">
+        <v>29312.7</v>
+      </c>
+      <c r="P31">
+        <v>28764.6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32">
+        <v>23.49</v>
+      </c>
+      <c r="C32">
+        <v>5.94</v>
+      </c>
+      <c r="D32">
+        <v>1.56</v>
+      </c>
+      <c r="G32" t="s">
+        <v>30</v>
+      </c>
+      <c r="H32">
+        <v>4264</v>
+      </c>
+      <c r="I32">
+        <v>16837</v>
+      </c>
+      <c r="J32">
+        <v>63919</v>
+      </c>
+      <c r="M32" t="s">
+        <v>30</v>
+      </c>
+      <c r="N32">
+        <v>29347.8</v>
+      </c>
+      <c r="O32">
+        <v>28641.4</v>
+      </c>
+      <c r="P32">
+        <v>28885.6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="B38" t="s">
+        <v>37</v>
+      </c>
+      <c r="C38" t="s">
+        <v>38</v>
+      </c>
+      <c r="D38" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" t="s">
+        <v>79</v>
+      </c>
+      <c r="C39" t="s">
+        <v>80</v>
+      </c>
+      <c r="D39" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" t="s">
+        <v>100</v>
+      </c>
+      <c r="D40" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41" t="s">
+        <v>102</v>
+      </c>
+      <c r="C41" t="s">
+        <v>103</v>
+      </c>
+      <c r="D41" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" t="s">
+        <v>105</v>
+      </c>
+      <c r="C42" t="s">
+        <v>106</v>
+      </c>
+      <c r="D42" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" t="s">
+        <v>57</v>
+      </c>
+      <c r="D43" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v0.17: top-stage extra spins (math re-simulated, all checks pass, bookcheck clean), Hacksaw-style big-win steps, TOTAL WIN screen, stage-up splash, multiplier flash fix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011QYnJU3qzdAzbD5jkFKhoX
</commit_message>
<xml_diff>
--- a/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
+++ b/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
@@ -141,49 +141,49 @@
     <t>{'symbol': 'scatter'}</t>
   </si>
   <si>
-    <t>9.89293193816642</t>
+    <t>9.892892480370161</t>
   </si>
   <si>
     <t>10094</t>
   </si>
   <si>
-    <t>97.47144368657537</t>
+    <t>96.86323897870895</t>
   </si>
   <si>
     <t>{'jaguar': '1'}</t>
   </si>
   <si>
-    <t>51.239338330852405</t>
+    <t>51.238570060773704</t>
   </si>
   <si>
     <t>1933</t>
   </si>
   <si>
-    <t>80.51459265391256</t>
+    <t>80.04832105955367</t>
   </si>
   <si>
     <t>{'jaguar': '2'}</t>
   </si>
   <si>
-    <t>80.25627539933097</t>
+    <t>80.25694310342968</t>
   </si>
   <si>
     <t>1257</t>
   </si>
   <si>
-    <t>99.54358661924113</t>
+    <t>99.54369901491287</t>
   </si>
   <si>
     <t>{'jaguar': '3'}</t>
   </si>
   <si>
-    <t>186.86176769661037</t>
+    <t>186.88114336727375</t>
   </si>
   <si>
     <t>535</t>
   </si>
   <si>
-    <t>100.55734001169911</t>
+    <t>106.06446529180673</t>
   </si>
   <si>
     <t>{'jaguar': '4'}</t>
@@ -192,40 +192,40 @@
     <t>0</t>
   </si>
   <si>
-    <t>4.007998232664069</t>
+    <t>4.008006183192583</t>
   </si>
   <si>
     <t>25200</t>
   </si>
   <si>
-    <t>148.27878465133733</t>
-  </si>
-  <si>
-    <t>53.695108810512416</t>
-  </si>
-  <si>
-    <t>1900</t>
-  </si>
-  <si>
-    <t>148.28901924751221</t>
-  </si>
-  <si>
-    <t>80.41797479258412</t>
+    <t>148.45179735605544</t>
+  </si>
+  <si>
+    <t>53.711713847325555</t>
+  </si>
+  <si>
+    <t>1899</t>
+  </si>
+  <si>
+    <t>144.25889414002637</t>
+  </si>
+  <si>
+    <t>80.41885983507716</t>
   </si>
   <si>
     <t>1277</t>
   </si>
   <si>
-    <t>147.40585780226954</t>
-  </si>
-  <si>
-    <t>197.2806933043873</t>
-  </si>
-  <si>
-    <t>513</t>
-  </si>
-  <si>
-    <t>133.6279173906405</t>
+    <t>148.11859979416005</t>
+  </si>
+  <si>
+    <t>197.53140843461034</t>
+  </si>
+  <si>
+    <t>512</t>
+  </si>
+  <si>
+    <t>129.09793176613076</t>
   </si>
   <si>
     <t>NaN</t>
@@ -264,94 +264,94 @@
     <t>100000</t>
   </si>
   <si>
-    <t>9600.000000405998</t>
-  </si>
-  <si>
-    <t>49.424038968972425</t>
+    <t>9600.00000073193</t>
+  </si>
+  <si>
+    <t>49.33834303870571</t>
   </si>
   <si>
     <t>2027</t>
   </si>
   <si>
-    <t>9151.893305175789</t>
-  </si>
-  <si>
-    <t>71.7970491953915</t>
+    <t>8747.126206698134</t>
+  </si>
+  <si>
+    <t>71.87603151707332</t>
   </si>
   <si>
     <t>1389</t>
   </si>
   <si>
-    <t>9997.404619714414</t>
-  </si>
-  <si>
-    <t>181.0788177540222</t>
+    <t>9694.812198045407</t>
+  </si>
+  <si>
+    <t>180.94881973589446</t>
   </si>
   <si>
     <t>552</t>
   </si>
   <si>
-    <t>8505.723482825519</t>
-  </si>
-  <si>
-    <t>19200.00000185894</t>
-  </si>
-  <si>
-    <t>48.710354215837334</t>
-  </si>
-  <si>
-    <t>2059</t>
-  </si>
-  <si>
-    <t>17916.26101670402</t>
-  </si>
-  <si>
-    <t>72.37983553395851</t>
-  </si>
-  <si>
-    <t>1384</t>
-  </si>
-  <si>
-    <t>20109.066909315286</t>
-  </si>
-  <si>
-    <t>165.70620759958825</t>
-  </si>
-  <si>
-    <t>610</t>
-  </si>
-  <si>
-    <t>15485.07618583011</t>
-  </si>
-  <si>
-    <t>48000.00000978044</t>
-  </si>
-  <si>
-    <t>48.63789443045843</t>
-  </si>
-  <si>
-    <t>2050</t>
-  </si>
-  <si>
-    <t>47739.229401464596</t>
-  </si>
-  <si>
-    <t>71.12275584802437</t>
-  </si>
-  <si>
-    <t>1400</t>
-  </si>
-  <si>
-    <t>47390.414822143866</t>
-  </si>
-  <si>
-    <t>186.37002731730232</t>
-  </si>
-  <si>
-    <t>538</t>
-  </si>
-  <si>
-    <t>46283.83577616291</t>
+    <t>9748.763877701851</t>
+  </si>
+  <si>
+    <t>19200.000000272194</t>
+  </si>
+  <si>
+    <t>48.58815606419479</t>
+  </si>
+  <si>
+    <t>2060</t>
+  </si>
+  <si>
+    <t>17883.17013082456</t>
+  </si>
+  <si>
+    <t>72.37289553058257</t>
+  </si>
+  <si>
+    <t>1385</t>
+  </si>
+  <si>
+    <t>19280.423181017926</t>
+  </si>
+  <si>
+    <t>164.700419110383</t>
+  </si>
+  <si>
+    <t>609</t>
+  </si>
+  <si>
+    <t>16787.74323577234</t>
+  </si>
+  <si>
+    <t>48000.000005110545</t>
+  </si>
+  <si>
+    <t>48.42224771315437</t>
+  </si>
+  <si>
+    <t>2056</t>
+  </si>
+  <si>
+    <t>46209.81306688033</t>
+  </si>
+  <si>
+    <t>70.5112617665084</t>
+  </si>
+  <si>
+    <t>1411</t>
+  </si>
+  <si>
+    <t>44645.97925324434</t>
+  </si>
+  <si>
+    <t>185.4664807552642</t>
+  </si>
+  <si>
+    <t>541</t>
+  </si>
+  <si>
+    <t>48433.63614053933</t>
   </si>
 </sst>
 </file>
@@ -731,7 +731,7 @@
         <v>6.716</v>
       </c>
       <c r="C3">
-        <v>0.07186539990587827</v>
+        <v>0.07187009181143961</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -740,7 +740,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>26873</v>
+        <v>26881</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -748,10 +748,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>16.568</v>
+        <v>16.566</v>
       </c>
       <c r="C4">
-        <v>0.07665465983507912</v>
+        <v>0.07666199105349815</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -760,7 +760,7 @@
         <v>5</v>
       </c>
       <c r="K4">
-        <v>11018</v>
+        <v>11017</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -768,10 +768,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>21.225</v>
+        <v>21.218</v>
       </c>
       <c r="C5">
-        <v>0.1360606550844265</v>
+        <v>0.1361111329943789</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -780,7 +780,7 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>9008</v>
+        <v>9009</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -788,10 +788,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>66.747</v>
+        <v>66.69</v>
       </c>
       <c r="C6">
-        <v>0.09741432971334846</v>
+        <v>0.0975010165665488</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -800,7 +800,7 @@
         <v>7</v>
       </c>
       <c r="K6">
-        <v>3624</v>
+        <v>3616</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -808,10 +808,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>158.254</v>
+        <v>157.846</v>
       </c>
       <c r="C7">
-        <v>0.08278113161179292</v>
+        <v>0.08299701454624574</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -820,7 +820,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>2584</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -828,10 +828,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>341.526</v>
+        <v>343.709</v>
       </c>
       <c r="C8">
-        <v>0.08739191522350541</v>
+        <v>0.08670934383331373</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -840,7 +840,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>2741</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -848,10 +848,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>926.414</v>
+        <v>951.891</v>
       </c>
       <c r="C9">
-        <v>0.0739950089064506</v>
+        <v>0.07205539526445708</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -860,7 +860,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>1637</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -868,10 +868,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>1739.106</v>
+        <v>1789.98</v>
       </c>
       <c r="C10">
-        <v>0.08135271798062613</v>
+        <v>0.07980209565157674</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -880,7 +880,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>1129</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -888,10 +888,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>4440.008</v>
+        <v>4320.97</v>
       </c>
       <c r="C11">
-        <v>0.05429144013312413</v>
+        <v>0.05598842836379844</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -900,7 +900,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>450</v>
+        <v>480</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -908,10 +908,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>5246.921</v>
+        <v>5490.871</v>
       </c>
       <c r="C12">
-        <v>0.07265553957752816</v>
+        <v>0.07001930628301455</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -928,10 +928,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>11728.888</v>
+        <v>11076.994</v>
       </c>
       <c r="C13">
-        <v>0.05852394369010371</v>
+        <v>0.06170205970340513</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -940,7 +940,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>308</v>
+        <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -948,10 +948,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>41614.592</v>
+        <v>38717.318</v>
       </c>
       <c r="C14">
-        <v>0.03195437913730449</v>
+        <v>0.0349652908607801</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -960,7 +960,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>111</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -968,10 +968,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>196432.869</v>
+        <v>159908.737</v>
       </c>
       <c r="C15">
-        <v>0.01216040265920396</v>
+        <v>0.01511689604910547</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -980,7 +980,7 @@
         <v>16</v>
       </c>
       <c r="K15">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -988,10 +988,10 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>368768.209</v>
+        <v>749510.064</v>
       </c>
       <c r="C16">
-        <v>0.01064273660693304</v>
+        <v>0.005162565798113454</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
@@ -1000,7 +1000,7 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -1008,10 +1008,10 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>1232686.609</v>
+        <v>896521.032</v>
       </c>
       <c r="C17">
-        <v>0.007216871704620448</v>
+        <v>0.006908752128176824</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -1020,7 +1020,7 @@
         <v>18</v>
       </c>
       <c r="K17">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -1028,10 +1028,10 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>2016589.27</v>
+        <v>2232601.338</v>
       </c>
       <c r="C18">
-        <v>0.004958875999120791</v>
+        <v>0.004479089699213472</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
@@ -1040,7 +1040,7 @@
         <v>19</v>
       </c>
       <c r="K18">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -1088,37 +1088,37 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>1471.37</v>
+        <v>1495.17</v>
       </c>
       <c r="C24">
-        <v>323.86</v>
+        <v>303.39</v>
       </c>
       <c r="D24">
-        <v>44.23</v>
+        <v>43.04</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I24">
-        <v>294</v>
+        <v>311</v>
       </c>
       <c r="J24">
-        <v>2285</v>
+        <v>2337</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>57.6</v>
+        <v>98.5</v>
       </c>
       <c r="O24">
-        <v>76.90000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="P24">
-        <v>100.1</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -1126,37 +1126,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>1456.92</v>
+        <v>1354.93</v>
       </c>
       <c r="C25">
-        <v>202.75</v>
+        <v>187.03</v>
       </c>
       <c r="D25">
-        <v>26.98</v>
+        <v>26.5</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I25">
-        <v>502</v>
+        <v>536</v>
       </c>
       <c r="J25">
-        <v>3633</v>
+        <v>3709</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>185.3</v>
+        <v>87.8</v>
       </c>
       <c r="O25">
-        <v>85.59999999999999</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="P25">
-        <v>86.7</v>
+        <v>86.5</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -1164,37 +1164,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>1280.67</v>
+        <v>1157.71</v>
       </c>
       <c r="C26">
-        <v>178.52</v>
+        <v>169.45</v>
       </c>
       <c r="D26">
-        <v>21.43</v>
+        <v>21.09</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="I26">
-        <v>549</v>
+        <v>579</v>
       </c>
       <c r="J26">
-        <v>4653</v>
+        <v>4732</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>73.90000000000001</v>
+        <v>63</v>
       </c>
       <c r="O26">
-        <v>87.59999999999999</v>
+        <v>88.8</v>
       </c>
       <c r="P26">
-        <v>91.40000000000001</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -1202,34 +1202,34 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>747.27</v>
+        <v>712.66</v>
       </c>
       <c r="C27">
-        <v>102.52</v>
+        <v>100.02</v>
       </c>
       <c r="D27">
-        <v>14.66</v>
+        <v>14.39</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="I27">
-        <v>964</v>
+        <v>990</v>
       </c>
       <c r="J27">
-        <v>6870</v>
+        <v>6989</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
-        <v>116.6</v>
+        <v>108.2</v>
       </c>
       <c r="O27">
-        <v>92.5</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="P27">
         <v>97.90000000000001</v>
@@ -1240,37 +1240,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>324.87</v>
+        <v>326.12</v>
       </c>
       <c r="C28">
-        <v>59.3</v>
+        <v>58.4</v>
       </c>
       <c r="D28">
-        <v>9.99</v>
+        <v>9.9</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="I28">
-        <v>1744</v>
+        <v>1767</v>
       </c>
       <c r="J28">
-        <v>9923</v>
+        <v>10023</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>98.90000000000001</v>
+        <v>96.3</v>
       </c>
       <c r="O28">
-        <v>98.7</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="P28">
-        <v>93.40000000000001</v>
+        <v>92.7</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -1278,37 +1278,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>195</v>
+        <v>192.36</v>
       </c>
       <c r="C29">
-        <v>41.76</v>
+        <v>41.06</v>
       </c>
       <c r="D29">
-        <v>8.01</v>
+        <v>7.94</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="I29">
-        <v>2361</v>
+        <v>2406</v>
       </c>
       <c r="J29">
-        <v>12456</v>
+        <v>12559</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>104.1</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="O29">
-        <v>97.3</v>
+        <v>96.2</v>
       </c>
       <c r="P29">
-        <v>96.8</v>
+        <v>94.5</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -1316,37 +1316,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>154.96</v>
+        <v>152.58</v>
       </c>
       <c r="C30">
-        <v>36.29</v>
+        <v>35.71</v>
       </c>
       <c r="D30">
-        <v>6.79</v>
+        <v>6.73</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>631</v>
+        <v>642</v>
       </c>
       <c r="I30">
-        <v>2777</v>
+        <v>2821</v>
       </c>
       <c r="J30">
-        <v>14731</v>
+        <v>14845</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>95.09999999999999</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="O30">
-        <v>111.4</v>
+        <v>109.7</v>
       </c>
       <c r="P30">
-        <v>100.9</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -1354,37 +1354,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>133.29</v>
+        <v>130.44</v>
       </c>
       <c r="C31">
-        <v>29.38</v>
+        <v>28.66</v>
       </c>
       <c r="D31">
-        <v>6.84</v>
+        <v>6.79</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>768</v>
+        <v>785</v>
       </c>
       <c r="I31">
-        <v>3368</v>
+        <v>3444</v>
       </c>
       <c r="J31">
-        <v>14612</v>
+        <v>14728</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>91</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="O31">
-        <v>95.2</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="P31">
-        <v>95.2</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -1392,37 +1392,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>123.6</v>
+        <v>121.09</v>
       </c>
       <c r="C32">
-        <v>30.36</v>
+        <v>29.87</v>
       </c>
       <c r="D32">
-        <v>6.61</v>
+        <v>6.58</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>830</v>
+        <v>845</v>
       </c>
       <c r="I32">
-        <v>3363</v>
+        <v>3419</v>
       </c>
       <c r="J32">
-        <v>15074</v>
+        <v>15151</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>113.9</v>
+        <v>105.9</v>
       </c>
       <c r="O32">
-        <v>96.8</v>
+        <v>98.7</v>
       </c>
       <c r="P32">
-        <v>95</v>
+        <v>95.2</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -1563,10 +1563,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>6.675</v>
+        <v>6.674</v>
       </c>
       <c r="C3">
-        <v>0.04825492153255811</v>
+        <v>0.04825992265294356</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -1575,7 +1575,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>24456</v>
+        <v>24467</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1583,10 +1583,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>16.684</v>
+        <v>16.681</v>
       </c>
       <c r="C4">
-        <v>0.05068681964521812</v>
+        <v>0.05069716543661059</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -1595,7 +1595,7 @@
         <v>5</v>
       </c>
       <c r="K4">
-        <v>10076</v>
+        <v>10072</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1603,10 +1603,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>21.119</v>
+        <v>21.106</v>
       </c>
       <c r="C5">
-        <v>0.09097619089354396</v>
+        <v>0.09103785400828059</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -1615,7 +1615,7 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>9034</v>
+        <v>9021</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1623,10 +1623,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>65.289</v>
+        <v>65.127</v>
       </c>
       <c r="C6">
-        <v>0.06664908070230434</v>
+        <v>0.06682969817965777</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -1635,7 +1635,7 @@
         <v>7</v>
       </c>
       <c r="K6">
-        <v>4914</v>
+        <v>4907</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1643,10 +1643,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>147.992</v>
+        <v>147.495</v>
       </c>
       <c r="C7">
-        <v>0.05962019734465319</v>
+        <v>0.05982952394468469</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -1655,7 +1655,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>4627</v>
+        <v>4599</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1663,10 +1663,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>224.582</v>
+        <v>226.148</v>
       </c>
       <c r="C8">
-        <v>0.09081335474024543</v>
+        <v>0.08995353142337713</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -1675,7 +1675,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>6532</v>
+        <v>6433</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1683,10 +1683,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>510.262</v>
+        <v>525.836</v>
       </c>
       <c r="C9">
-        <v>0.09021663783253574</v>
+        <v>0.08738278915716201</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -1695,7 +1695,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>4249</v>
+        <v>4165</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1703,10 +1703,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>874.434</v>
+        <v>917.59</v>
       </c>
       <c r="C10">
-        <v>0.1072135890410191</v>
+        <v>0.1023057772005038</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -1715,7 +1715,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>2845</v>
+        <v>2795</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1723,10 +1723,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>2337.594</v>
+        <v>2397.698</v>
       </c>
       <c r="C11">
-        <v>0.06973810730949261</v>
+        <v>0.06766838069638863</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -1735,7 +1735,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>1070</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1743,10 +1743,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>2856.483</v>
+        <v>2670.858</v>
       </c>
       <c r="C12">
-        <v>0.08944651160960206</v>
+        <v>0.09607257941011905</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -1755,7 +1755,7 @@
         <v>13</v>
       </c>
       <c r="K12">
-        <v>909</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1763,10 +1763,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>5359.855</v>
+        <v>5001.817</v>
       </c>
       <c r="C13">
-        <v>0.08589465744373981</v>
+        <v>0.09113324103267224</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -1775,7 +1775,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>701</v>
+        <v>805</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1783,10 +1783,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>15683.287</v>
+        <v>15658.137</v>
       </c>
       <c r="C14">
-        <v>0.05671885075069664</v>
+        <v>0.05668724319608853</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -1795,7 +1795,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>286</v>
+        <v>312</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1803,10 +1803,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>82617.17200000001</v>
+        <v>86655.223</v>
       </c>
       <c r="C15">
-        <v>0.01912645634936879</v>
+        <v>0.01873329680312645</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -1815,7 +1815,7 @@
         <v>16</v>
       </c>
       <c r="K15">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1823,10 +1823,10 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>153009.107</v>
+        <v>176753.965</v>
       </c>
       <c r="C16">
-        <v>0.01631794638151567</v>
+        <v>0.01406669888064927</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
@@ -1835,7 +1835,7 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -1843,10 +1843,10 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>387398.874</v>
+        <v>404808.296</v>
       </c>
       <c r="C17">
-        <v>0.01164340323360451</v>
+        <v>0.01088997109722522</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -1855,7 +1855,7 @@
         <v>18</v>
       </c>
       <c r="K17">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -1863,10 +1863,10 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>1011131.34</v>
+        <v>932365.287</v>
       </c>
       <c r="C18">
-        <v>0.006593284332536043</v>
+        <v>0.007150280600193694</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
@@ -1875,7 +1875,7 @@
         <v>19</v>
       </c>
       <c r="K18">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -1923,37 +1923,37 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>849.1</v>
+        <v>917.03</v>
       </c>
       <c r="C24">
-        <v>172.82</v>
+        <v>167.43</v>
       </c>
       <c r="D24">
-        <v>21.97</v>
+        <v>21.33</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="I24">
-        <v>600</v>
+        <v>614</v>
       </c>
       <c r="J24">
-        <v>4611</v>
+        <v>4741</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>116</v>
+        <v>171.6</v>
       </c>
       <c r="O24">
-        <v>189.5</v>
+        <v>156.7</v>
       </c>
       <c r="P24">
-        <v>142.7</v>
+        <v>140.6</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -1961,37 +1961,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>777.13</v>
+        <v>759.05</v>
       </c>
       <c r="C25">
-        <v>106.76</v>
+        <v>101.52</v>
       </c>
       <c r="D25">
-        <v>14.47</v>
+        <v>14.21</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I25">
-        <v>981</v>
+        <v>1040</v>
       </c>
       <c r="J25">
-        <v>7088</v>
+        <v>7263</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>152.9</v>
+        <v>142.1</v>
       </c>
       <c r="O25">
-        <v>135.4</v>
+        <v>138.7</v>
       </c>
       <c r="P25">
-        <v>154.7</v>
+        <v>153.1</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -1999,37 +1999,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>703.14</v>
+        <v>659.74</v>
       </c>
       <c r="C26">
-        <v>93.97</v>
+        <v>90.98</v>
       </c>
       <c r="D26">
-        <v>13.2</v>
+        <v>12.9</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="I26">
-        <v>1045</v>
+        <v>1090</v>
       </c>
       <c r="J26">
-        <v>7648</v>
+        <v>7836</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>152</v>
+        <v>153.8</v>
       </c>
       <c r="O26">
-        <v>153.9</v>
+        <v>133.2</v>
       </c>
       <c r="P26">
-        <v>145</v>
+        <v>140.6</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -2037,37 +2037,37 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>401.27</v>
+        <v>383.35</v>
       </c>
       <c r="C27">
-        <v>56.58</v>
+        <v>54.49</v>
       </c>
       <c r="D27">
-        <v>8.41</v>
+        <v>8.26</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="I27">
-        <v>1737</v>
+        <v>1800</v>
       </c>
       <c r="J27">
-        <v>11911</v>
+        <v>12138</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
+        <v>131.9</v>
+      </c>
+      <c r="O27">
         <v>148</v>
       </c>
-      <c r="O27">
-        <v>147.9</v>
-      </c>
       <c r="P27">
-        <v>150.5</v>
+        <v>151.4</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -2075,37 +2075,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>192.81</v>
+        <v>187.29</v>
       </c>
       <c r="C28">
-        <v>36.51</v>
+        <v>35.51</v>
       </c>
       <c r="D28">
-        <v>6.19</v>
+        <v>6.12</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>534</v>
+        <v>553</v>
       </c>
       <c r="I28">
-        <v>2762</v>
+        <v>2842</v>
       </c>
       <c r="J28">
-        <v>16096</v>
+        <v>16317</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>144.1</v>
+        <v>146.6</v>
       </c>
       <c r="O28">
-        <v>156.2</v>
+        <v>158</v>
       </c>
       <c r="P28">
-        <v>148</v>
+        <v>148.4</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -2113,37 +2113,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>125.02</v>
+        <v>120.46</v>
       </c>
       <c r="C29">
-        <v>26.64</v>
+        <v>26.12</v>
       </c>
       <c r="D29">
-        <v>5.35</v>
+        <v>5.29</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>754</v>
+        <v>782</v>
       </c>
       <c r="I29">
-        <v>3784</v>
+        <v>3869</v>
       </c>
       <c r="J29">
-        <v>18641</v>
+        <v>18870</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>142.4</v>
+        <v>152.4</v>
       </c>
       <c r="O29">
-        <v>146.6</v>
+        <v>145.9</v>
       </c>
       <c r="P29">
-        <v>146.5</v>
+        <v>145.4</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -2151,37 +2151,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>103.52</v>
+        <v>101.02</v>
       </c>
       <c r="C30">
-        <v>22.38</v>
+        <v>21.88</v>
       </c>
       <c r="D30">
-        <v>4.74</v>
+        <v>4.69</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>1009</v>
+        <v>1040</v>
       </c>
       <c r="I30">
-        <v>4391</v>
+        <v>4522</v>
       </c>
       <c r="J30">
-        <v>21267</v>
+        <v>21541</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>145.2</v>
+        <v>143.2</v>
       </c>
       <c r="O30">
-        <v>135.4</v>
+        <v>136</v>
       </c>
       <c r="P30">
-        <v>140.3</v>
+        <v>141.3</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -2189,37 +2189,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>69.13</v>
+        <v>67.72</v>
       </c>
       <c r="C31">
-        <v>17.18</v>
+        <v>16.83</v>
       </c>
       <c r="D31">
-        <v>4.32</v>
+        <v>4.28</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>1446</v>
+        <v>1488</v>
       </c>
       <c r="I31">
-        <v>5885</v>
+        <v>6009</v>
       </c>
       <c r="J31">
-        <v>23463</v>
+        <v>23693</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>131.7</v>
+        <v>133.9</v>
       </c>
       <c r="O31">
-        <v>146.6</v>
+        <v>152.1</v>
       </c>
       <c r="P31">
-        <v>149.4</v>
+        <v>152.3</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2227,37 +2227,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>69.01000000000001</v>
+        <v>67.33</v>
       </c>
       <c r="C32">
-        <v>17.31</v>
+        <v>16.91</v>
       </c>
       <c r="D32">
-        <v>4.18</v>
+        <v>4.15</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>1434</v>
+        <v>1478</v>
       </c>
       <c r="I32">
-        <v>5833</v>
+        <v>5971</v>
       </c>
       <c r="J32">
-        <v>24068</v>
+        <v>24259</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>145.4</v>
+        <v>129.8</v>
       </c>
       <c r="O32">
-        <v>147</v>
+        <v>144.3</v>
       </c>
       <c r="P32">
-        <v>144.1</v>
+        <v>144.8</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -3233,10 +3233,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>95.65900000000001</v>
+        <v>84.852</v>
       </c>
       <c r="C3">
-        <v>5.589167660799064E-05</v>
+        <v>6.29180606176708E-05</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -3245,7 +3245,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>1300</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -3253,10 +3253,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>61.629</v>
+        <v>55.892</v>
       </c>
       <c r="C4">
-        <v>0.0002285440672368884</v>
+        <v>0.0002516780196369835</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -3265,7 +3265,7 @@
         <v>5</v>
       </c>
       <c r="K4">
-        <v>1954</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -3273,10 +3273,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>16.869</v>
+        <v>15.602</v>
       </c>
       <c r="C5">
-        <v>0.002034829462151282</v>
+        <v>0.002194909365315611</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -3285,7 +3285,7 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>6844</v>
+        <v>6812</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -3293,10 +3293,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>9.754</v>
+        <v>9.260999999999999</v>
       </c>
       <c r="C6">
-        <v>0.007566113530902545</v>
+        <v>0.007957604417342454</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -3305,7 +3305,7 @@
         <v>7</v>
       </c>
       <c r="K6">
-        <v>11311</v>
+        <v>11250</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -3313,10 +3313,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>6.217</v>
+        <v>6.064</v>
       </c>
       <c r="C7">
-        <v>0.0234986314945006</v>
+        <v>0.02405356491061927</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -3325,7 +3325,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>16987</v>
+        <v>16854</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -3333,10 +3333,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>3.884</v>
+        <v>3.939</v>
       </c>
       <c r="C8">
-        <v>0.08399638775377694</v>
+        <v>0.08249634021839182</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -3345,7 +3345,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>25781</v>
+        <v>25349</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -3353,10 +3353,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>5.982</v>
+        <v>6.302</v>
       </c>
       <c r="C9">
-        <v>0.1186141038050749</v>
+        <v>0.1123375858020789</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -3365,7 +3365,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>15849</v>
+        <v>15468</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -3373,10 +3373,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>8.872999999999999</v>
+        <v>9.523999999999999</v>
       </c>
       <c r="C10">
-        <v>0.1584294158200309</v>
+        <v>0.1476340937813647</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -3385,7 +3385,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>10186</v>
+        <v>10023</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -3393,10 +3393,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>23.68</v>
+        <v>24.279</v>
       </c>
       <c r="C11">
-        <v>0.1029939749122851</v>
+        <v>0.1003701709734936</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -3405,7 +3405,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>3668</v>
+        <v>3864</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -3413,10 +3413,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>27.507</v>
+        <v>26.871</v>
       </c>
       <c r="C12">
-        <v>0.1391156373920316</v>
+        <v>0.1428339896189153</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -3425,7 +3425,7 @@
         <v>13</v>
       </c>
       <c r="K12">
-        <v>3060</v>
+        <v>3443</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -3433,10 +3433,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>38.611</v>
+        <v>35.032</v>
       </c>
       <c r="C13">
-        <v>0.1766459207944776</v>
+        <v>0.1946115401658967</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -3445,7 +3445,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>2094</v>
+        <v>2595</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -3453,10 +3453,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>143.249</v>
+        <v>139.863</v>
       </c>
       <c r="C14">
-        <v>0.09278292348794855</v>
+        <v>0.09436304948821864</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -3465,7 +3465,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>673</v>
+        <v>796</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -3473,10 +3473,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>848.434</v>
+        <v>859.975</v>
       </c>
       <c r="C15">
-        <v>0.02790040253787059</v>
+        <v>0.02818969075813448</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -3485,7 +3485,7 @@
         <v>16</v>
       </c>
       <c r="K15">
-        <v>109</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -3493,10 +3493,10 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>1642.429</v>
+        <v>2081.014</v>
       </c>
       <c r="C16">
-        <v>0.02116407731417595</v>
+        <v>0.0166800786526409</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
@@ -3505,7 +3505,7 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -3513,10 +3513,10 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>19154.868</v>
+        <v>16056.017</v>
       </c>
       <c r="C17">
-        <v>0.003395114141437955</v>
+        <v>0.004027418240386174</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -3525,7 +3525,7 @@
         <v>18</v>
       </c>
       <c r="K17">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -3533,10 +3533,10 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>86678.55499999999</v>
+        <v>62177.683</v>
       </c>
       <c r="C18">
-        <v>0.001153689900005999</v>
+        <v>0.001608297080104057</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
@@ -3545,7 +3545,7 @@
         <v>19</v>
       </c>
       <c r="K18">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -3593,13 +3593,13 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>325.71</v>
+        <v>325.27</v>
       </c>
       <c r="C24">
-        <v>53.35</v>
+        <v>51.18</v>
       </c>
       <c r="D24">
-        <v>6.52</v>
+        <v>6.36</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
@@ -3608,22 +3608,22 @@
         <v>308</v>
       </c>
       <c r="I24">
-        <v>1870</v>
+        <v>1953</v>
       </c>
       <c r="J24">
-        <v>15348</v>
+        <v>15731</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>9754.1</v>
+        <v>9996.1</v>
       </c>
       <c r="O24">
-        <v>9226.6</v>
+        <v>9548.700000000001</v>
       </c>
       <c r="P24">
-        <v>9285.9</v>
+        <v>9337.9</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -3631,37 +3631,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>231.23</v>
+        <v>220.65</v>
       </c>
       <c r="C25">
-        <v>31.41</v>
+        <v>30.33</v>
       </c>
       <c r="D25">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>435</v>
+        <v>454</v>
       </c>
       <c r="I25">
-        <v>3182</v>
+        <v>3299</v>
       </c>
       <c r="J25">
-        <v>22749</v>
+        <v>23246</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>9099.1</v>
+        <v>9332.299999999999</v>
       </c>
       <c r="O25">
-        <v>10026.9</v>
+        <v>9962</v>
       </c>
       <c r="P25">
-        <v>9587.700000000001</v>
+        <v>9540.5</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -3669,37 +3669,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>215.28</v>
+        <v>206.78</v>
       </c>
       <c r="C26">
-        <v>30.85</v>
+        <v>29.85</v>
       </c>
       <c r="D26">
-        <v>4.51</v>
+        <v>4.41</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>462</v>
+        <v>482</v>
       </c>
       <c r="I26">
-        <v>3241</v>
+        <v>3350</v>
       </c>
       <c r="J26">
-        <v>22139</v>
+        <v>22670</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>9930.299999999999</v>
+        <v>10124.3</v>
       </c>
       <c r="O26">
-        <v>9946.1</v>
+        <v>9962.200000000001</v>
       </c>
       <c r="P26">
-        <v>9771.200000000001</v>
+        <v>9790.299999999999</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -3707,37 +3707,37 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>113.25</v>
+        <v>110.47</v>
       </c>
       <c r="C27">
-        <v>17.8</v>
+        <v>17.32</v>
       </c>
       <c r="D27">
-        <v>2.84</v>
+        <v>2.79</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>880</v>
+        <v>903</v>
       </c>
       <c r="I27">
-        <v>5619</v>
+        <v>5775</v>
       </c>
       <c r="J27">
-        <v>35185</v>
+        <v>35877</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
-        <v>9831.5</v>
+        <v>10157.8</v>
       </c>
       <c r="O27">
-        <v>10075.1</v>
+        <v>9864.799999999999</v>
       </c>
       <c r="P27">
-        <v>9541.9</v>
+        <v>9640.299999999999</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -3745,37 +3745,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>62.88</v>
+        <v>61.09</v>
       </c>
       <c r="C28">
-        <v>12.67</v>
+        <v>12.34</v>
       </c>
       <c r="D28">
-        <v>2.34</v>
+        <v>2.3</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>1601</v>
+        <v>1644</v>
       </c>
       <c r="I28">
-        <v>7897</v>
+        <v>8107</v>
       </c>
       <c r="J28">
-        <v>42739</v>
+        <v>43504</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>9278.700000000001</v>
+        <v>9310.9</v>
       </c>
       <c r="O28">
-        <v>9353.299999999999</v>
+        <v>9470.6</v>
       </c>
       <c r="P28">
-        <v>9491.6</v>
+        <v>9557.4</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -3783,37 +3783,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>46.16</v>
+        <v>44.48</v>
       </c>
       <c r="C29">
-        <v>9.609999999999999</v>
+        <v>9.34</v>
       </c>
       <c r="D29">
-        <v>2.15</v>
+        <v>2.12</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>2164</v>
+        <v>2247</v>
       </c>
       <c r="I29">
-        <v>10413</v>
+        <v>10708</v>
       </c>
       <c r="J29">
-        <v>46412</v>
+        <v>47156</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>9783.1</v>
+        <v>9552.200000000001</v>
       </c>
       <c r="O29">
-        <v>9263.299999999999</v>
+        <v>9246.1</v>
       </c>
       <c r="P29">
-        <v>9634.799999999999</v>
+        <v>9615.200000000001</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -3821,37 +3821,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>34.52</v>
+        <v>33.49</v>
       </c>
       <c r="C30">
-        <v>8.52</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="D30">
-        <v>2.01</v>
+        <v>1.98</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>2891</v>
+        <v>2981</v>
       </c>
       <c r="I30">
-        <v>11747</v>
+        <v>12082</v>
       </c>
       <c r="J30">
-        <v>49774</v>
+        <v>50563</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>8914.700000000001</v>
+        <v>8954.9</v>
       </c>
       <c r="O30">
-        <v>9545.5</v>
+        <v>9632</v>
       </c>
       <c r="P30">
-        <v>9632.700000000001</v>
+        <v>9656.799999999999</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -3859,37 +3859,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>24.18</v>
+        <v>23.4</v>
       </c>
       <c r="C31">
-        <v>5.67</v>
+        <v>5.52</v>
       </c>
       <c r="D31">
-        <v>1.55</v>
+        <v>1.53</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>4135</v>
+        <v>4275</v>
       </c>
       <c r="I31">
-        <v>17625</v>
+        <v>18095</v>
       </c>
       <c r="J31">
-        <v>64527</v>
+        <v>65246</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>10042.7</v>
+        <v>9952</v>
       </c>
       <c r="O31">
-        <v>9700.299999999999</v>
+        <v>9672</v>
       </c>
       <c r="P31">
-        <v>9567.1</v>
+        <v>9599.700000000001</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -3897,37 +3897,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>21.58</v>
+        <v>20.97</v>
       </c>
       <c r="C32">
-        <v>5.56</v>
+        <v>5.42</v>
       </c>
       <c r="D32">
-        <v>1.52</v>
+        <v>1.51</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>4645</v>
+        <v>4774</v>
       </c>
       <c r="I32">
-        <v>18010</v>
+        <v>18448</v>
       </c>
       <c r="J32">
-        <v>65742</v>
+        <v>66289</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>9497.9</v>
+        <v>9577.299999999999</v>
       </c>
       <c r="O32">
-        <v>9518.9</v>
+        <v>9587</v>
       </c>
       <c r="P32">
-        <v>9676.700000000001</v>
+        <v>9645.5</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -4068,10 +4068,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>168.231</v>
+        <v>139.189</v>
       </c>
       <c r="C3">
-        <v>1.461905706378885E-05</v>
+        <v>1.763736663715365E-05</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -4080,7 +4080,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>927</v>
+        <v>882</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -4088,10 +4088,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>158.588</v>
+        <v>134.109</v>
       </c>
       <c r="C4">
-        <v>4.346590369999947E-05</v>
+        <v>5.129709179558277E-05</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -4100,7 +4100,7 @@
         <v>5</v>
       </c>
       <c r="K4">
-        <v>932</v>
+        <v>893</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -4108,10 +4108,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>52.088</v>
+        <v>45.837</v>
       </c>
       <c r="C5">
-        <v>0.0003256842812694324</v>
+        <v>0.0003682431181267729</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -4120,7 +4120,7 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>2651</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4128,10 +4128,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>28.876</v>
+        <v>26.261</v>
       </c>
       <c r="C6">
-        <v>0.001271799118633527</v>
+        <v>0.001396498931104341</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -4140,7 +4140,7 @@
         <v>7</v>
       </c>
       <c r="K6">
-        <v>4443</v>
+        <v>4271</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -4148,10 +4148,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>13.219</v>
+        <v>12.518</v>
       </c>
       <c r="C7">
-        <v>0.005565044835517494</v>
+        <v>0.005863532381818695</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -4160,7 +4160,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>9034</v>
+        <v>8668</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -4168,10 +4168,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>5.07</v>
+        <v>5.073</v>
       </c>
       <c r="C8">
-        <v>0.03348302164507189</v>
+        <v>0.03334721082805956</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -4180,7 +4180,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>21545</v>
+        <v>20526</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -4188,10 +4188,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>4.75</v>
+        <v>4.968</v>
       </c>
       <c r="C9">
-        <v>0.07572868620439716</v>
+        <v>0.07230878265613899</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -4200,7 +4200,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>21122</v>
+        <v>20149</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -4208,10 +4208,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>5.227</v>
+        <v>5.491</v>
       </c>
       <c r="C10">
-        <v>0.1358703140830078</v>
+        <v>0.1298369575485657</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -4220,7 +4220,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>17780</v>
+        <v>17590</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -4228,10 +4228,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>11.193</v>
+        <v>11.35</v>
       </c>
       <c r="C11">
-        <v>0.1091414966900078</v>
+        <v>0.1079438597793559</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -4240,7 +4240,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>7797</v>
+        <v>8266</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -4248,10 +4248,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>12.112</v>
+        <v>11.668</v>
       </c>
       <c r="C12">
-        <v>0.1580674011027271</v>
+        <v>0.1654360009365402</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -4260,7 +4260,7 @@
         <v>13</v>
       </c>
       <c r="K12">
-        <v>6852</v>
+        <v>7853</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -4268,10 +4268,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>16.032</v>
+        <v>15.16</v>
       </c>
       <c r="C13">
-        <v>0.2145184094044471</v>
+        <v>0.2262540611400718</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -4280,7 +4280,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>4849</v>
+        <v>5867</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -4288,10 +4288,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>53.628</v>
+        <v>50.246</v>
       </c>
       <c r="C14">
-        <v>0.1241348602626982</v>
+        <v>0.1330826915922397</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -4300,7 +4300,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>1494</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -4308,10 +4308,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>270.031</v>
+        <v>306.181</v>
       </c>
       <c r="C15">
-        <v>0.04459083430824589</v>
+        <v>0.03919091450880752</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -4320,7 +4320,7 @@
         <v>16</v>
       </c>
       <c r="K15">
-        <v>277</v>
+        <v>302</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -4328,10 +4328,10 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>513.754</v>
+        <v>646.466</v>
       </c>
       <c r="C16">
-        <v>0.03536651368809048</v>
+        <v>0.02796007699025207</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
@@ -4340,7 +4340,7 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -4348,10 +4348,10 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>1660.608</v>
+        <v>2022.996</v>
       </c>
       <c r="C17">
-        <v>0.01966512751801837</v>
+        <v>0.01528874517898457</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -4360,7 +4360,7 @@
         <v>18</v>
       </c>
       <c r="K17">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -4368,10 +4368,10 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>24868.064</v>
+        <v>36752.644</v>
       </c>
       <c r="C18">
-        <v>0.002010632772307765</v>
+        <v>0.001360455471374746</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
@@ -4428,37 +4428,37 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>320.69</v>
+        <v>313.64</v>
       </c>
       <c r="C24">
-        <v>54.09</v>
+        <v>50.22</v>
       </c>
       <c r="D24">
-        <v>6.73</v>
+        <v>6.31</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="I24">
-        <v>1844</v>
+        <v>1991</v>
       </c>
       <c r="J24">
-        <v>14899</v>
+        <v>15870</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>26787.6</v>
+        <v>20824.5</v>
       </c>
       <c r="O24">
-        <v>20392</v>
+        <v>19626.3</v>
       </c>
       <c r="P24">
-        <v>19135.3</v>
+        <v>19109.5</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -4466,37 +4466,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>236.9</v>
+        <v>220.91</v>
       </c>
       <c r="C25">
-        <v>32.13</v>
+        <v>29.52</v>
       </c>
       <c r="D25">
-        <v>4.59</v>
+        <v>4.32</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>417</v>
+        <v>450</v>
       </c>
       <c r="I25">
-        <v>3119</v>
+        <v>3391</v>
       </c>
       <c r="J25">
-        <v>21784</v>
+        <v>23147</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>20644</v>
+        <v>20305.6</v>
       </c>
       <c r="O25">
-        <v>19655.9</v>
+        <v>19276.4</v>
       </c>
       <c r="P25">
-        <v>18999.1</v>
+        <v>18838.7</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -4504,37 +4504,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>242.74</v>
+        <v>220.77</v>
       </c>
       <c r="C26">
-        <v>32</v>
+        <v>29.78</v>
       </c>
       <c r="D26">
-        <v>4.72</v>
+        <v>4.43</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>407</v>
+        <v>450</v>
       </c>
       <c r="I26">
-        <v>3111</v>
+        <v>3352</v>
       </c>
       <c r="J26">
-        <v>21183</v>
+        <v>22565</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>19348.5</v>
+        <v>20409.1</v>
       </c>
       <c r="O26">
-        <v>19893.6</v>
+        <v>19680.4</v>
       </c>
       <c r="P26">
-        <v>19346.3</v>
+        <v>19404.7</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -4542,37 +4542,37 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>117.77</v>
+        <v>110.16</v>
       </c>
       <c r="C27">
-        <v>17.77</v>
+        <v>16.64</v>
       </c>
       <c r="D27">
-        <v>2.85</v>
+        <v>2.71</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>850</v>
+        <v>908</v>
       </c>
       <c r="I27">
-        <v>5618</v>
+        <v>6006</v>
       </c>
       <c r="J27">
-        <v>35101</v>
+        <v>36850</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
-        <v>19962.4</v>
+        <v>20366.4</v>
       </c>
       <c r="O27">
-        <v>19999.6</v>
+        <v>19688.9</v>
       </c>
       <c r="P27">
-        <v>19135.9</v>
+        <v>19137.5</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -4580,37 +4580,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>63.8</v>
+        <v>60.18</v>
       </c>
       <c r="C28">
-        <v>12.74</v>
+        <v>11.99</v>
       </c>
       <c r="D28">
-        <v>2.32</v>
+        <v>2.22</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>1569</v>
+        <v>1666</v>
       </c>
       <c r="I28">
-        <v>7867</v>
+        <v>8349</v>
       </c>
       <c r="J28">
-        <v>43063</v>
+        <v>45116</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>19839.7</v>
+        <v>19779.8</v>
       </c>
       <c r="O28">
-        <v>19559.5</v>
+        <v>19229.6</v>
       </c>
       <c r="P28">
-        <v>19276.8</v>
+        <v>19341.9</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -4618,37 +4618,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>47.59</v>
+        <v>44.33</v>
       </c>
       <c r="C29">
-        <v>9.99</v>
+        <v>9.31</v>
       </c>
       <c r="D29">
-        <v>2.23</v>
+        <v>2.13</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>2092</v>
+        <v>2253</v>
       </c>
       <c r="I29">
-        <v>10017</v>
+        <v>10747</v>
       </c>
       <c r="J29">
-        <v>44840</v>
+        <v>46885</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>20218.7</v>
+        <v>19884.7</v>
       </c>
       <c r="O29">
-        <v>18973.3</v>
+        <v>18979</v>
       </c>
       <c r="P29">
-        <v>19309.6</v>
+        <v>19249.2</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -4656,37 +4656,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>37.09</v>
+        <v>34.38</v>
       </c>
       <c r="C30">
-        <v>8.859999999999999</v>
+        <v>8.32</v>
       </c>
       <c r="D30">
-        <v>2.09</v>
+        <v>2</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>2709</v>
+        <v>2913</v>
       </c>
       <c r="I30">
-        <v>11297</v>
+        <v>12030</v>
       </c>
       <c r="J30">
-        <v>47910</v>
+        <v>50025</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>17462.6</v>
+        <v>17244.1</v>
       </c>
       <c r="O30">
-        <v>19500.8</v>
+        <v>19476.6</v>
       </c>
       <c r="P30">
-        <v>19258</v>
+        <v>19198.1</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -4694,37 +4694,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>24.62</v>
+        <v>22.79</v>
       </c>
       <c r="C31">
-        <v>5.91</v>
+        <v>5.53</v>
       </c>
       <c r="D31">
-        <v>1.6</v>
+        <v>1.54</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>4059</v>
+        <v>4385</v>
       </c>
       <c r="I31">
-        <v>16937</v>
+        <v>18101</v>
       </c>
       <c r="J31">
-        <v>62662</v>
+        <v>64766</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>19308.9</v>
+        <v>19908.7</v>
       </c>
       <c r="O31">
-        <v>19530.7</v>
+        <v>19349.2</v>
       </c>
       <c r="P31">
-        <v>19089.4</v>
+        <v>19162.9</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -4732,37 +4732,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>22.73</v>
+        <v>21.21</v>
       </c>
       <c r="C32">
-        <v>5.75</v>
+        <v>5.4</v>
       </c>
       <c r="D32">
-        <v>1.52</v>
+        <v>1.48</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>4404</v>
+        <v>4717</v>
       </c>
       <c r="I32">
-        <v>17447</v>
+        <v>18524</v>
       </c>
       <c r="J32">
-        <v>65683</v>
+        <v>67421</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>19121.9</v>
+        <v>19389.3</v>
       </c>
       <c r="O32">
-        <v>18995.2</v>
+        <v>19033.9</v>
       </c>
       <c r="P32">
-        <v>19116</v>
+        <v>19122.4</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -4903,10 +4903,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>36.541</v>
+        <v>30.168</v>
       </c>
       <c r="C3">
-        <v>2.595893244453806E-05</v>
+        <v>3.130506781332828E-05</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -4915,7 +4915,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>1130</v>
+        <v>2071</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -4923,10 +4923,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>56.062</v>
+        <v>54.284</v>
       </c>
       <c r="C4">
-        <v>4.805233395972363E-05</v>
+        <v>4.938686577061096E-05</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -4935,7 +4935,7 @@
         <v>5</v>
       </c>
       <c r="K4">
-        <v>801</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -4943,10 +4943,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>40.088</v>
+        <v>35.039</v>
       </c>
       <c r="C5">
-        <v>0.0001566786597993961</v>
+        <v>0.000180492827362639</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -4955,7 +4955,7 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>1237</v>
+        <v>1976</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4963,10 +4963,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>41.833</v>
+        <v>33.485</v>
       </c>
       <c r="C6">
-        <v>0.0003364018872838057</v>
+        <v>0.0004194468537812072</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -4975,7 +4975,7 @@
         <v>7</v>
       </c>
       <c r="K6">
-        <v>1336</v>
+        <v>2209</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -4983,10 +4983,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>24.502</v>
+        <v>19.648</v>
       </c>
       <c r="C7">
-        <v>0.001141156534920645</v>
+        <v>0.001416775437222132</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -4995,7 +4995,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>2549</v>
+        <v>4004</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -5003,10 +5003,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>10.352</v>
+        <v>9.034000000000001</v>
       </c>
       <c r="C8">
-        <v>0.006403380013688451</v>
+        <v>0.007310835927315079</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -5015,7 +5015,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>6976</v>
+        <v>9442</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -5023,10 +5023,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>8.74</v>
+        <v>8.281000000000001</v>
       </c>
       <c r="C9">
-        <v>0.01666751766005454</v>
+        <v>0.01748041623111436</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -5035,7 +5035,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>9505</v>
+        <v>11135</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -5043,10 +5043,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>6.557</v>
+        <v>6.74</v>
       </c>
       <c r="C10">
-        <v>0.04418341737472563</v>
+        <v>0.04287579577376968</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -5055,7 +5055,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>14310</v>
+        <v>14647</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -5063,10 +5063,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>9.896000000000001</v>
+        <v>10.965</v>
       </c>
       <c r="C11">
-        <v>0.04976248109889216</v>
+        <v>0.04474447006650164</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -5075,7 +5075,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>10440</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -5083,10 +5083,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>7.933</v>
+        <v>9.19</v>
       </c>
       <c r="C12">
-        <v>0.0979895405247691</v>
+        <v>0.08487320527402402</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -5095,7 +5095,7 @@
         <v>13</v>
       </c>
       <c r="K12">
-        <v>14120</v>
+        <v>11866</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -5103,10 +5103,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>7.024</v>
+        <v>7.896</v>
       </c>
       <c r="C13">
-        <v>0.201479184653081</v>
+        <v>0.1794116187600719</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -5115,7 +5115,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>17725</v>
+        <v>14643</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -5123,10 +5123,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>11.553</v>
+        <v>12.242</v>
       </c>
       <c r="C14">
-        <v>0.2392663172343997</v>
+        <v>0.2273911526925453</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -5135,7 +5135,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>12146</v>
+        <v>10103</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -5143,10 +5143,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>38.924</v>
+        <v>37.359</v>
       </c>
       <c r="C15">
-        <v>0.1237745767145003</v>
+        <v>0.1298278517320922</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -5155,7 +5155,7 @@
         <v>16</v>
       </c>
       <c r="K15">
-        <v>3989</v>
+        <v>3503</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -5163,10 +5163,10 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>68.425</v>
+        <v>58.936</v>
       </c>
       <c r="C16">
-        <v>0.1096784911279149</v>
+        <v>0.1275543823075197</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
@@ -5175,7 +5175,7 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>2455</v>
+        <v>2319</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -5183,10 +5183,10 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>192.806</v>
+        <v>139.335</v>
       </c>
       <c r="C17">
-        <v>0.06775005172515892</v>
+        <v>0.09498666906946536</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -5195,7 +5195,7 @@
         <v>18</v>
       </c>
       <c r="K17">
-        <v>961</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -5203,10 +5203,10 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>16212.166</v>
+        <v>15159.773</v>
       </c>
       <c r="C18">
-        <v>0.001233650965274922</v>
+        <v>0.001319293056230302</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
@@ -5215,7 +5215,7 @@
         <v>19</v>
       </c>
       <c r="K18">
-        <v>320</v>
+        <v>339</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -5263,37 +5263,37 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>413.35</v>
+        <v>440.71</v>
       </c>
       <c r="C24">
-        <v>61.07</v>
+        <v>66.47</v>
       </c>
       <c r="D24">
-        <v>7.3</v>
+        <v>7.85</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="I24">
-        <v>1646</v>
+        <v>1515</v>
       </c>
       <c r="J24">
-        <v>13718</v>
+        <v>12734</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>51621.7</v>
+        <v>53191.8</v>
       </c>
       <c r="O24">
-        <v>48862.8</v>
+        <v>51155.3</v>
       </c>
       <c r="P24">
-        <v>47871.8</v>
+        <v>47748.9</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -5301,37 +5301,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>263.17</v>
+        <v>289.38</v>
       </c>
       <c r="C25">
-        <v>35.34</v>
+        <v>38.32</v>
       </c>
       <c r="D25">
-        <v>4.98</v>
+        <v>5.39</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>388</v>
+        <v>350</v>
       </c>
       <c r="I25">
-        <v>2803</v>
+        <v>2606</v>
       </c>
       <c r="J25">
-        <v>20091</v>
+        <v>18559</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>52145.5</v>
+        <v>47784.7</v>
       </c>
       <c r="O25">
-        <v>46289.1</v>
+        <v>47576</v>
       </c>
       <c r="P25">
-        <v>48164.4</v>
+        <v>48367.2</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -5339,37 +5339,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>265.84</v>
+        <v>287.02</v>
       </c>
       <c r="C26">
-        <v>34.99</v>
+        <v>37.23</v>
       </c>
       <c r="D26">
-        <v>5.13</v>
+        <v>5.52</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>386</v>
+        <v>352</v>
       </c>
       <c r="I26">
-        <v>2869</v>
+        <v>2678</v>
       </c>
       <c r="J26">
-        <v>19471</v>
+        <v>18088</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>47295.5</v>
+        <v>47162.1</v>
       </c>
       <c r="O26">
-        <v>50373.3</v>
+        <v>48922.2</v>
       </c>
       <c r="P26">
-        <v>47628.6</v>
+        <v>47488</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -5377,37 +5377,37 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>134.42</v>
+        <v>149.69</v>
       </c>
       <c r="C27">
-        <v>18.44</v>
+        <v>19.28</v>
       </c>
       <c r="D27">
-        <v>2.84</v>
+        <v>3</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>737</v>
+        <v>674</v>
       </c>
       <c r="I27">
-        <v>5431</v>
+        <v>5194</v>
       </c>
       <c r="J27">
-        <v>35163</v>
+        <v>33344</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
-        <v>45796.7</v>
+        <v>51259.5</v>
       </c>
       <c r="O27">
-        <v>48433.6</v>
+        <v>50236.4</v>
       </c>
       <c r="P27">
-        <v>47750.6</v>
+        <v>47698.1</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -5415,37 +5415,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>64.09999999999999</v>
+        <v>68.39</v>
       </c>
       <c r="C28">
-        <v>13.02</v>
+        <v>13.81</v>
       </c>
       <c r="D28">
-        <v>2.36</v>
+        <v>2.47</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>1562</v>
+        <v>1462</v>
       </c>
       <c r="I28">
-        <v>7669</v>
+        <v>7251</v>
       </c>
       <c r="J28">
-        <v>42445</v>
+        <v>40464</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>47939.9</v>
+        <v>45833.6</v>
       </c>
       <c r="O28">
-        <v>48157.2</v>
+        <v>49493.8</v>
       </c>
       <c r="P28">
-        <v>47986</v>
+        <v>48030.7</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -5453,37 +5453,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>53.21</v>
+        <v>58.12</v>
       </c>
       <c r="C29">
-        <v>10.89</v>
+        <v>11.69</v>
       </c>
       <c r="D29">
-        <v>2.39</v>
+        <v>2.56</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>1869</v>
+        <v>1717</v>
       </c>
       <c r="I29">
-        <v>9184</v>
+        <v>8562</v>
       </c>
       <c r="J29">
-        <v>41929</v>
+        <v>39103</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>48264.1</v>
+        <v>49364.1</v>
       </c>
       <c r="O29">
-        <v>47972.6</v>
+        <v>47890.3</v>
       </c>
       <c r="P29">
-        <v>47982.9</v>
+        <v>47521.4</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -5491,37 +5491,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>43.31</v>
+        <v>46.72</v>
       </c>
       <c r="C30">
-        <v>10.48</v>
+        <v>11.23</v>
       </c>
       <c r="D30">
-        <v>2.37</v>
+        <v>2.52</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>2301</v>
+        <v>2141</v>
       </c>
       <c r="I30">
-        <v>9574</v>
+        <v>8910</v>
       </c>
       <c r="J30">
-        <v>42265</v>
+        <v>39575</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>47287.6</v>
+        <v>47548.5</v>
       </c>
       <c r="O30">
-        <v>48236.5</v>
+        <v>47744.3</v>
       </c>
       <c r="P30">
-        <v>47963</v>
+        <v>47777.2</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -5529,37 +5529,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>26.7</v>
+        <v>28.46</v>
       </c>
       <c r="C31">
-        <v>6.36</v>
+        <v>6.8</v>
       </c>
       <c r="D31">
-        <v>1.68</v>
+        <v>1.78</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>3744</v>
+        <v>3506</v>
       </c>
       <c r="I31">
-        <v>15763</v>
+        <v>14724</v>
       </c>
       <c r="J31">
-        <v>59613</v>
+        <v>56181</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>47578.4</v>
+        <v>47755.7</v>
       </c>
       <c r="O31">
-        <v>48552.4</v>
+        <v>48732.4</v>
       </c>
       <c r="P31">
-        <v>48065.3</v>
+        <v>48094.5</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -5567,37 +5567,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>24.85</v>
+        <v>26.98</v>
       </c>
       <c r="C32">
-        <v>6.15</v>
+        <v>6.63</v>
       </c>
       <c r="D32">
-        <v>1.56</v>
+        <v>1.66</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>4023</v>
+        <v>3719</v>
       </c>
       <c r="I32">
-        <v>16188</v>
+        <v>15066</v>
       </c>
       <c r="J32">
-        <v>64309</v>
+        <v>60387</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>48676.9</v>
+        <v>47789.9</v>
       </c>
       <c r="O32">
-        <v>47205</v>
+        <v>47494.6</v>
       </c>
       <c r="P32">
-        <v>48084.4</v>
+        <v>47843.2</v>
       </c>
     </row>
     <row r="37" spans="1:4">

</xml_diff>

<commit_message>
Jaguar King feature spin (200x, king steles 50-500x), new BONUS symbol (step pyramid), name BALAM RISING
</commit_message>
<xml_diff>
--- a/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
+++ b/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
@@ -10,16 +10,17 @@
     <sheet name="base" sheetId="1" r:id="rId1"/>
     <sheet name="bonushunt" sheetId="2" r:id="rId2"/>
     <sheet name="jaguar" sheetId="3" r:id="rId3"/>
-    <sheet name="bonus" sheetId="4" r:id="rId4"/>
-    <sheet name="superbonus" sheetId="5" r:id="rId5"/>
-    <sheet name="godbonus" sheetId="6" r:id="rId6"/>
+    <sheet name="jaguarking" sheetId="4" r:id="rId4"/>
+    <sheet name="bonus" sheetId="5" r:id="rId5"/>
+    <sheet name="superbonus" sheetId="6" r:id="rId6"/>
+    <sheet name="godbonus" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="117">
   <si>
     <t>Win Ranges</t>
   </si>
@@ -256,6 +257,24 @@
   </si>
   <si>
     <t>2385.1646356552055</t>
+  </si>
+  <si>
+    <t>2.0033775890958276</t>
+  </si>
+  <si>
+    <t>19217.340703473896</t>
+  </si>
+  <si>
+    <t>2.9797571339862867</t>
+  </si>
+  <si>
+    <t>19240.94819954831</t>
+  </si>
+  <si>
+    <t>6.051614714775488</t>
+  </si>
+  <si>
+    <t>19064.456788819545</t>
   </si>
   <si>
     <t>1.0</t>
@@ -3232,11 +3251,11 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3">
-        <v>84.852</v>
+      <c r="B3" t="s">
+        <v>69</v>
       </c>
       <c r="C3">
-        <v>6.29180606176708E-05</v>
+        <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -3245,18 +3264,18 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>1294</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
-        <v>55.892</v>
+      <c r="B4" t="s">
+        <v>69</v>
       </c>
       <c r="C4">
-        <v>0.0002516780196369835</v>
+        <v>0</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -3265,18 +3284,18 @@
         <v>5</v>
       </c>
       <c r="K4">
-        <v>1937</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5">
-        <v>15.602</v>
+      <c r="B5" t="s">
+        <v>69</v>
       </c>
       <c r="C5">
-        <v>0.002194909365315611</v>
+        <v>0</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -3285,18 +3304,18 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>6812</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
-        <v>9.260999999999999</v>
+      <c r="B6" t="s">
+        <v>69</v>
       </c>
       <c r="C6">
-        <v>0.007957604417342454</v>
+        <v>0</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -3305,18 +3324,18 @@
         <v>7</v>
       </c>
       <c r="K6">
-        <v>11250</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B7">
-        <v>6.064</v>
+      <c r="B7" t="s">
+        <v>69</v>
       </c>
       <c r="C7">
-        <v>0.02405356491061927</v>
+        <v>0</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -3325,7 +3344,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>16854</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -3333,10 +3352,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>3.939</v>
+        <v>5.693</v>
       </c>
       <c r="C8">
-        <v>0.08249634021839182</v>
+        <v>0.03023891102145014</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -3345,7 +3364,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>25349</v>
+        <v>17403</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -3353,10 +3372,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>6.302</v>
+        <v>3.862</v>
       </c>
       <c r="C9">
-        <v>0.1123375858020789</v>
+        <v>0.09066130701457091</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -3365,7 +3384,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>15468</v>
+        <v>25791</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -3373,10 +3392,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>9.523999999999999</v>
+        <v>3.542</v>
       </c>
       <c r="C10">
-        <v>0.1476340937813647</v>
+        <v>0.1922369331082189</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -3385,7 +3404,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>10023</v>
+        <v>28256</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -3393,10 +3412,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>24.279</v>
+        <v>8.654</v>
       </c>
       <c r="C11">
-        <v>0.1003701709734936</v>
+        <v>0.1354056206207358</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -3405,7 +3424,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>3864</v>
+        <v>11613</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -3413,10 +3432,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>26.871</v>
+        <v>10.222</v>
       </c>
       <c r="C12">
-        <v>0.1428339896189153</v>
+        <v>0.1816094882657492</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -3425,7 +3444,7 @@
         <v>13</v>
       </c>
       <c r="K12">
-        <v>3443</v>
+        <v>9865</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -3433,10 +3452,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>35.032</v>
+        <v>19.619</v>
       </c>
       <c r="C13">
-        <v>0.1946115401658967</v>
+        <v>0.1704128380538051</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -3445,7 +3464,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>2595</v>
+        <v>5162</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -3453,10 +3472,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>139.863</v>
+        <v>68.173</v>
       </c>
       <c r="C14">
-        <v>0.09436304948821864</v>
+        <v>0.09616335272235986</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -3465,7 +3484,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>796</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -3473,10 +3492,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>859.975</v>
+        <v>407.256</v>
       </c>
       <c r="C15">
-        <v>0.02818969075813448</v>
+        <v>0.02835934303822878</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -3485,7 +3504,7 @@
         <v>16</v>
       </c>
       <c r="K15">
-        <v>127</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -3493,10 +3512,10 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>2081.014</v>
+        <v>801.259</v>
       </c>
       <c r="C16">
-        <v>0.0166800786526409</v>
+        <v>0.02267627180529015</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
@@ -3505,7 +3524,7 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>61</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -3513,10 +3532,10 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>16056.017</v>
+        <v>2861.043</v>
       </c>
       <c r="C17">
-        <v>0.004027418240386174</v>
+        <v>0.01126830047061499</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -3525,7 +3544,7 @@
         <v>18</v>
       </c>
       <c r="K17">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -3533,10 +3552,10 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>62177.683</v>
+        <v>51672.431</v>
       </c>
       <c r="C18">
-        <v>0.001608297080104057</v>
+        <v>0.000967633970204461</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
@@ -3545,7 +3564,7 @@
         <v>19</v>
       </c>
       <c r="K18">
-        <v>105</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -3593,37 +3612,37 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>325.27</v>
+        <v>33259.08</v>
       </c>
       <c r="C24">
-        <v>51.18</v>
+        <v>951.84</v>
       </c>
       <c r="D24">
-        <v>6.36</v>
+        <v>66.81999999999999</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24">
-        <v>308</v>
+        <v>3</v>
       </c>
       <c r="I24">
-        <v>1953</v>
+        <v>105</v>
       </c>
       <c r="J24">
-        <v>15731</v>
+        <v>1496</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>9996.1</v>
+        <v>9324.6</v>
       </c>
       <c r="O24">
-        <v>9548.700000000001</v>
+        <v>16862.1</v>
       </c>
       <c r="P24">
-        <v>9337.9</v>
+        <v>18667.8</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -3631,37 +3650,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>220.65</v>
+        <v>6645.09</v>
       </c>
       <c r="C25">
-        <v>30.33</v>
+        <v>454.9</v>
       </c>
       <c r="D25">
-        <v>4.3</v>
+        <v>38.14</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>454</v>
+        <v>15</v>
       </c>
       <c r="I25">
-        <v>3299</v>
+        <v>220</v>
       </c>
       <c r="J25">
-        <v>23246</v>
+        <v>2622</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>9332.299999999999</v>
+        <v>10299.3</v>
       </c>
       <c r="O25">
-        <v>9962</v>
+        <v>21426</v>
       </c>
       <c r="P25">
-        <v>9540.5</v>
+        <v>18274.9</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -3669,37 +3688,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>206.78</v>
+        <v>2130.69</v>
       </c>
       <c r="C26">
-        <v>29.85</v>
+        <v>246.88</v>
       </c>
       <c r="D26">
-        <v>4.41</v>
+        <v>21.79</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>482</v>
+        <v>47</v>
       </c>
       <c r="I26">
-        <v>3350</v>
+        <v>405</v>
       </c>
       <c r="J26">
-        <v>22670</v>
+        <v>4590</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>10124.3</v>
+        <v>20614.8</v>
       </c>
       <c r="O26">
-        <v>9962.200000000001</v>
+        <v>18041.2</v>
       </c>
       <c r="P26">
-        <v>9790.299999999999</v>
+        <v>20074.7</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -3707,37 +3726,37 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>110.47</v>
+        <v>1351.57</v>
       </c>
       <c r="C27">
-        <v>17.32</v>
+        <v>154.87</v>
       </c>
       <c r="D27">
-        <v>2.79</v>
+        <v>15.42</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>903</v>
+        <v>74</v>
       </c>
       <c r="I27">
-        <v>5775</v>
+        <v>646</v>
       </c>
       <c r="J27">
-        <v>35877</v>
+        <v>6484</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
-        <v>10157.8</v>
+        <v>20884.4</v>
       </c>
       <c r="O27">
-        <v>9864.799999999999</v>
+        <v>20882.1</v>
       </c>
       <c r="P27">
-        <v>9640.299999999999</v>
+        <v>19187.5</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -3745,37 +3764,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>61.09</v>
+        <v>469.08</v>
       </c>
       <c r="C28">
-        <v>12.34</v>
+        <v>66.93000000000001</v>
       </c>
       <c r="D28">
-        <v>2.3</v>
+        <v>8.9</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>1644</v>
+        <v>213</v>
       </c>
       <c r="I28">
-        <v>8107</v>
+        <v>1494</v>
       </c>
       <c r="J28">
-        <v>43504</v>
+        <v>11234</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>9310.9</v>
+        <v>16892</v>
       </c>
       <c r="O28">
-        <v>9470.6</v>
+        <v>19703.3</v>
       </c>
       <c r="P28">
-        <v>9557.4</v>
+        <v>19696.9</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -3783,37 +3802,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>44.48</v>
+        <v>303.83</v>
       </c>
       <c r="C29">
-        <v>9.34</v>
+        <v>44.39</v>
       </c>
       <c r="D29">
-        <v>2.12</v>
+        <v>6.52</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>2247</v>
+        <v>329</v>
       </c>
       <c r="I29">
-        <v>10708</v>
+        <v>2253</v>
       </c>
       <c r="J29">
-        <v>47156</v>
+        <v>15337</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>9552.200000000001</v>
+        <v>17688.7</v>
       </c>
       <c r="O29">
-        <v>9246.1</v>
+        <v>18841.8</v>
       </c>
       <c r="P29">
-        <v>9615.200000000001</v>
+        <v>19372.9</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -3821,37 +3840,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>33.49</v>
+        <v>238.04</v>
       </c>
       <c r="C30">
-        <v>8.279999999999999</v>
+        <v>37.31</v>
       </c>
       <c r="D30">
-        <v>1.98</v>
+        <v>5.21</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>2981</v>
+        <v>420</v>
       </c>
       <c r="I30">
-        <v>12082</v>
+        <v>2681</v>
       </c>
       <c r="J30">
-        <v>50563</v>
+        <v>19189</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>8954.9</v>
+        <v>17797.5</v>
       </c>
       <c r="O30">
-        <v>9632</v>
+        <v>20006.3</v>
       </c>
       <c r="P30">
-        <v>9656.799999999999</v>
+        <v>19265.2</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -3859,37 +3878,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>23.4</v>
+        <v>178.19</v>
       </c>
       <c r="C31">
-        <v>5.52</v>
+        <v>34.81</v>
       </c>
       <c r="D31">
-        <v>1.53</v>
+        <v>5.79</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>4275</v>
+        <v>561</v>
       </c>
       <c r="I31">
-        <v>18095</v>
+        <v>2873</v>
       </c>
       <c r="J31">
-        <v>65246</v>
+        <v>17259</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>9952</v>
+        <v>16830</v>
       </c>
       <c r="O31">
-        <v>9672</v>
+        <v>19290.5</v>
       </c>
       <c r="P31">
-        <v>9599.700000000001</v>
+        <v>18845.6</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -3897,37 +3916,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>20.97</v>
+        <v>216.84</v>
       </c>
       <c r="C32">
-        <v>5.42</v>
+        <v>38.55</v>
       </c>
       <c r="D32">
-        <v>1.51</v>
+        <v>5.95</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>4774</v>
+        <v>461</v>
       </c>
       <c r="I32">
-        <v>18448</v>
+        <v>2594</v>
       </c>
       <c r="J32">
-        <v>66289</v>
+        <v>16819</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>9577.299999999999</v>
+        <v>17889.5</v>
       </c>
       <c r="O32">
-        <v>9587</v>
+        <v>18550.2</v>
       </c>
       <c r="P32">
-        <v>9645.5</v>
+        <v>19039.8</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -3951,13 +3970,13 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="C39" t="s">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="D39" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -3965,13 +3984,13 @@
         <v>43</v>
       </c>
       <c r="B40" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="C40" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="D40" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -3979,13 +3998,13 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C41" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="D41" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -3993,13 +4012,13 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C42" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="D42" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -4007,13 +4026,13 @@
         <v>55</v>
       </c>
       <c r="B43" t="s">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="C43" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="D43" t="s">
-        <v>56</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -4068,10 +4087,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>139.189</v>
+        <v>84.852</v>
       </c>
       <c r="C3">
-        <v>1.763736663715365E-05</v>
+        <v>6.29180606176708E-05</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -4080,7 +4099,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>882</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -4088,10 +4107,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>134.109</v>
+        <v>55.892</v>
       </c>
       <c r="C4">
-        <v>5.129709179558277E-05</v>
+        <v>0.0002516780196369835</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -4100,7 +4119,7 @@
         <v>5</v>
       </c>
       <c r="K4">
-        <v>893</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -4108,10 +4127,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>45.837</v>
+        <v>15.602</v>
       </c>
       <c r="C5">
-        <v>0.0003682431181267729</v>
+        <v>0.002194909365315611</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -4120,7 +4139,7 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>2532</v>
+        <v>6812</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4128,10 +4147,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>26.261</v>
+        <v>9.260999999999999</v>
       </c>
       <c r="C6">
-        <v>0.001396498931104341</v>
+        <v>0.007957604417342454</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -4140,7 +4159,7 @@
         <v>7</v>
       </c>
       <c r="K6">
-        <v>4271</v>
+        <v>11250</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -4148,10 +4167,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>12.518</v>
+        <v>6.064</v>
       </c>
       <c r="C7">
-        <v>0.005863532381818695</v>
+        <v>0.02405356491061927</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -4160,7 +4179,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>8668</v>
+        <v>16854</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -4168,10 +4187,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>5.073</v>
+        <v>3.939</v>
       </c>
       <c r="C8">
-        <v>0.03334721082805956</v>
+        <v>0.08249634021839182</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -4180,7 +4199,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>20526</v>
+        <v>25349</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -4188,10 +4207,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>4.968</v>
+        <v>6.302</v>
       </c>
       <c r="C9">
-        <v>0.07230878265613899</v>
+        <v>0.1123375858020789</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -4200,7 +4219,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>20149</v>
+        <v>15468</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -4208,10 +4227,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>5.491</v>
+        <v>9.523999999999999</v>
       </c>
       <c r="C10">
-        <v>0.1298369575485657</v>
+        <v>0.1476340937813647</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -4220,7 +4239,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>17590</v>
+        <v>10023</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -4228,10 +4247,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>11.35</v>
+        <v>24.279</v>
       </c>
       <c r="C11">
-        <v>0.1079438597793559</v>
+        <v>0.1003701709734936</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -4240,7 +4259,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>8266</v>
+        <v>3864</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -4248,10 +4267,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>11.668</v>
+        <v>26.871</v>
       </c>
       <c r="C12">
-        <v>0.1654360009365402</v>
+        <v>0.1428339896189153</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -4260,7 +4279,7 @@
         <v>13</v>
       </c>
       <c r="K12">
-        <v>7853</v>
+        <v>3443</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -4268,10 +4287,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>15.16</v>
+        <v>35.032</v>
       </c>
       <c r="C13">
-        <v>0.2262540611400718</v>
+        <v>0.1946115401658967</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -4280,7 +4299,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>5867</v>
+        <v>2595</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -4288,10 +4307,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>50.246</v>
+        <v>139.863</v>
       </c>
       <c r="C14">
-        <v>0.1330826915922397</v>
+        <v>0.09436304948821864</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -4300,7 +4319,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>1899</v>
+        <v>796</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -4308,10 +4327,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>306.181</v>
+        <v>859.975</v>
       </c>
       <c r="C15">
-        <v>0.03919091450880752</v>
+        <v>0.02818969075813448</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -4320,7 +4339,7 @@
         <v>16</v>
       </c>
       <c r="K15">
-        <v>302</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -4328,10 +4347,10 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>646.466</v>
+        <v>2081.014</v>
       </c>
       <c r="C16">
-        <v>0.02796007699025207</v>
+        <v>0.0166800786526409</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
@@ -4340,7 +4359,7 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>140</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -4348,10 +4367,10 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>2022.996</v>
+        <v>16056.017</v>
       </c>
       <c r="C17">
-        <v>0.01528874517898457</v>
+        <v>0.004027418240386174</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -4360,7 +4379,7 @@
         <v>18</v>
       </c>
       <c r="K17">
-        <v>51</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -4368,10 +4387,10 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>36752.644</v>
+        <v>62177.683</v>
       </c>
       <c r="C18">
-        <v>0.001360455471374746</v>
+        <v>0.001608297080104057</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
@@ -4380,7 +4399,7 @@
         <v>19</v>
       </c>
       <c r="K18">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -4428,37 +4447,37 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>313.64</v>
+        <v>325.27</v>
       </c>
       <c r="C24">
-        <v>50.22</v>
+        <v>51.18</v>
       </c>
       <c r="D24">
-        <v>6.31</v>
+        <v>6.36</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="I24">
-        <v>1991</v>
+        <v>1953</v>
       </c>
       <c r="J24">
-        <v>15870</v>
+        <v>15731</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>20824.5</v>
+        <v>9996.1</v>
       </c>
       <c r="O24">
-        <v>19626.3</v>
+        <v>9548.700000000001</v>
       </c>
       <c r="P24">
-        <v>19109.5</v>
+        <v>9337.9</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -4466,37 +4485,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>220.91</v>
+        <v>220.65</v>
       </c>
       <c r="C25">
-        <v>29.52</v>
+        <v>30.33</v>
       </c>
       <c r="D25">
-        <v>4.32</v>
+        <v>4.3</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="I25">
-        <v>3391</v>
+        <v>3299</v>
       </c>
       <c r="J25">
-        <v>23147</v>
+        <v>23246</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>20305.6</v>
+        <v>9332.299999999999</v>
       </c>
       <c r="O25">
-        <v>19276.4</v>
+        <v>9962</v>
       </c>
       <c r="P25">
-        <v>18838.7</v>
+        <v>9540.5</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -4504,37 +4523,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>220.77</v>
+        <v>206.78</v>
       </c>
       <c r="C26">
-        <v>29.78</v>
+        <v>29.85</v>
       </c>
       <c r="D26">
-        <v>4.43</v>
+        <v>4.41</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>450</v>
+        <v>482</v>
       </c>
       <c r="I26">
-        <v>3352</v>
+        <v>3350</v>
       </c>
       <c r="J26">
-        <v>22565</v>
+        <v>22670</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>20409.1</v>
+        <v>10124.3</v>
       </c>
       <c r="O26">
-        <v>19680.4</v>
+        <v>9962.200000000001</v>
       </c>
       <c r="P26">
-        <v>19404.7</v>
+        <v>9790.299999999999</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -4542,37 +4561,37 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>110.16</v>
+        <v>110.47</v>
       </c>
       <c r="C27">
-        <v>16.64</v>
+        <v>17.32</v>
       </c>
       <c r="D27">
-        <v>2.71</v>
+        <v>2.79</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="I27">
-        <v>6006</v>
+        <v>5775</v>
       </c>
       <c r="J27">
-        <v>36850</v>
+        <v>35877</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
-        <v>20366.4</v>
+        <v>10157.8</v>
       </c>
       <c r="O27">
-        <v>19688.9</v>
+        <v>9864.799999999999</v>
       </c>
       <c r="P27">
-        <v>19137.5</v>
+        <v>9640.299999999999</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -4580,37 +4599,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>60.18</v>
+        <v>61.09</v>
       </c>
       <c r="C28">
-        <v>11.99</v>
+        <v>12.34</v>
       </c>
       <c r="D28">
-        <v>2.22</v>
+        <v>2.3</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>1666</v>
+        <v>1644</v>
       </c>
       <c r="I28">
-        <v>8349</v>
+        <v>8107</v>
       </c>
       <c r="J28">
-        <v>45116</v>
+        <v>43504</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>19779.8</v>
+        <v>9310.9</v>
       </c>
       <c r="O28">
-        <v>19229.6</v>
+        <v>9470.6</v>
       </c>
       <c r="P28">
-        <v>19341.9</v>
+        <v>9557.4</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -4618,37 +4637,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>44.33</v>
+        <v>44.48</v>
       </c>
       <c r="C29">
-        <v>9.31</v>
+        <v>9.34</v>
       </c>
       <c r="D29">
-        <v>2.13</v>
+        <v>2.12</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>2253</v>
+        <v>2247</v>
       </c>
       <c r="I29">
-        <v>10747</v>
+        <v>10708</v>
       </c>
       <c r="J29">
-        <v>46885</v>
+        <v>47156</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>19884.7</v>
+        <v>9552.200000000001</v>
       </c>
       <c r="O29">
-        <v>18979</v>
+        <v>9246.1</v>
       </c>
       <c r="P29">
-        <v>19249.2</v>
+        <v>9615.200000000001</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -4656,37 +4675,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>34.38</v>
+        <v>33.49</v>
       </c>
       <c r="C30">
-        <v>8.32</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="D30">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>2913</v>
+        <v>2981</v>
       </c>
       <c r="I30">
-        <v>12030</v>
+        <v>12082</v>
       </c>
       <c r="J30">
-        <v>50025</v>
+        <v>50563</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>17244.1</v>
+        <v>8954.9</v>
       </c>
       <c r="O30">
-        <v>19476.6</v>
+        <v>9632</v>
       </c>
       <c r="P30">
-        <v>19198.1</v>
+        <v>9656.799999999999</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -4694,37 +4713,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>22.79</v>
+        <v>23.4</v>
       </c>
       <c r="C31">
-        <v>5.53</v>
+        <v>5.52</v>
       </c>
       <c r="D31">
-        <v>1.54</v>
+        <v>1.53</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>4385</v>
+        <v>4275</v>
       </c>
       <c r="I31">
-        <v>18101</v>
+        <v>18095</v>
       </c>
       <c r="J31">
-        <v>64766</v>
+        <v>65246</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>19908.7</v>
+        <v>9952</v>
       </c>
       <c r="O31">
-        <v>19349.2</v>
+        <v>9672</v>
       </c>
       <c r="P31">
-        <v>19162.9</v>
+        <v>9599.700000000001</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -4732,37 +4751,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>21.21</v>
+        <v>20.97</v>
       </c>
       <c r="C32">
-        <v>5.4</v>
+        <v>5.42</v>
       </c>
       <c r="D32">
-        <v>1.48</v>
+        <v>1.51</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>4717</v>
+        <v>4774</v>
       </c>
       <c r="I32">
-        <v>18524</v>
+        <v>18448</v>
       </c>
       <c r="J32">
-        <v>67421</v>
+        <v>66289</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>19389.3</v>
+        <v>9577.299999999999</v>
       </c>
       <c r="O32">
-        <v>19033.9</v>
+        <v>9587</v>
       </c>
       <c r="P32">
-        <v>19122.4</v>
+        <v>9645.5</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -4786,13 +4805,13 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="C39" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D39" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -4800,13 +4819,13 @@
         <v>43</v>
       </c>
       <c r="B40" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C40" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D40" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -4814,13 +4833,13 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C41" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D41" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -4828,13 +4847,13 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C42" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D42" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -4903,10 +4922,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>30.168</v>
+        <v>139.189</v>
       </c>
       <c r="C3">
-        <v>3.130506781332828E-05</v>
+        <v>1.763736663715365E-05</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -4915,7 +4934,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>2071</v>
+        <v>882</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -4923,10 +4942,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>54.284</v>
+        <v>134.109</v>
       </c>
       <c r="C4">
-        <v>4.938686577061096E-05</v>
+        <v>5.129709179558277E-05</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -4935,7 +4954,7 @@
         <v>5</v>
       </c>
       <c r="K4">
-        <v>1206</v>
+        <v>893</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -4943,10 +4962,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>35.039</v>
+        <v>45.837</v>
       </c>
       <c r="C5">
-        <v>0.000180492827362639</v>
+        <v>0.0003682431181267729</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -4955,7 +4974,7 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>1976</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4963,10 +4982,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>33.485</v>
+        <v>26.261</v>
       </c>
       <c r="C6">
-        <v>0.0004194468537812072</v>
+        <v>0.001396498931104341</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -4975,7 +4994,7 @@
         <v>7</v>
       </c>
       <c r="K6">
-        <v>2209</v>
+        <v>4271</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -4983,10 +5002,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>19.648</v>
+        <v>12.518</v>
       </c>
       <c r="C7">
-        <v>0.001416775437222132</v>
+        <v>0.005863532381818695</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -4995,7 +5014,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>4004</v>
+        <v>8668</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -5003,10 +5022,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>9.034000000000001</v>
+        <v>5.073</v>
       </c>
       <c r="C8">
-        <v>0.007310835927315079</v>
+        <v>0.03334721082805956</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -5015,7 +5034,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>9442</v>
+        <v>20526</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -5023,10 +5042,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>8.281000000000001</v>
+        <v>4.968</v>
       </c>
       <c r="C9">
-        <v>0.01748041623111436</v>
+        <v>0.07230878265613899</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -5035,7 +5054,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>11135</v>
+        <v>20149</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -5043,10 +5062,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>6.74</v>
+        <v>5.491</v>
       </c>
       <c r="C10">
-        <v>0.04287579577376968</v>
+        <v>0.1298369575485657</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -5055,7 +5074,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>14647</v>
+        <v>17590</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -5063,10 +5082,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>10.965</v>
+        <v>11.35</v>
       </c>
       <c r="C11">
-        <v>0.04474447006650164</v>
+        <v>0.1079438597793559</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -5075,7 +5094,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>9500</v>
+        <v>8266</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -5083,10 +5102,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>9.19</v>
+        <v>11.668</v>
       </c>
       <c r="C12">
-        <v>0.08487320527402402</v>
+        <v>0.1654360009365402</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -5095,7 +5114,7 @@
         <v>13</v>
       </c>
       <c r="K12">
-        <v>11866</v>
+        <v>7853</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -5103,10 +5122,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>7.896</v>
+        <v>15.16</v>
       </c>
       <c r="C13">
-        <v>0.1794116187600719</v>
+        <v>0.2262540611400718</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -5115,7 +5134,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>14643</v>
+        <v>5867</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -5123,10 +5142,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>12.242</v>
+        <v>50.246</v>
       </c>
       <c r="C14">
-        <v>0.2273911526925453</v>
+        <v>0.1330826915922397</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -5135,7 +5154,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>10103</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -5143,10 +5162,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>37.359</v>
+        <v>306.181</v>
       </c>
       <c r="C15">
-        <v>0.1298278517320922</v>
+        <v>0.03919091450880752</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -5155,7 +5174,7 @@
         <v>16</v>
       </c>
       <c r="K15">
-        <v>3503</v>
+        <v>302</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -5163,10 +5182,10 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>58.936</v>
+        <v>646.466</v>
       </c>
       <c r="C16">
-        <v>0.1275543823075197</v>
+        <v>0.02796007699025207</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
@@ -5175,7 +5194,7 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>2319</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -5183,10 +5202,10 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>139.335</v>
+        <v>2022.996</v>
       </c>
       <c r="C17">
-        <v>0.09498666906946536</v>
+        <v>0.01528874517898457</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -5195,7 +5214,7 @@
         <v>18</v>
       </c>
       <c r="K17">
-        <v>1037</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -5203,10 +5222,10 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>15159.773</v>
+        <v>36752.644</v>
       </c>
       <c r="C18">
-        <v>0.001319293056230302</v>
+        <v>0.001360455471374746</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
@@ -5215,7 +5234,7 @@
         <v>19</v>
       </c>
       <c r="K18">
-        <v>339</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -5263,37 +5282,37 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>440.71</v>
+        <v>313.64</v>
       </c>
       <c r="C24">
-        <v>66.47</v>
+        <v>50.22</v>
       </c>
       <c r="D24">
-        <v>7.85</v>
+        <v>6.31</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24">
-        <v>226</v>
+        <v>320</v>
       </c>
       <c r="I24">
-        <v>1515</v>
+        <v>1991</v>
       </c>
       <c r="J24">
-        <v>12734</v>
+        <v>15870</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>53191.8</v>
+        <v>20824.5</v>
       </c>
       <c r="O24">
-        <v>51155.3</v>
+        <v>19626.3</v>
       </c>
       <c r="P24">
-        <v>47748.9</v>
+        <v>19109.5</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -5301,37 +5320,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>289.38</v>
+        <v>220.91</v>
       </c>
       <c r="C25">
-        <v>38.32</v>
+        <v>29.52</v>
       </c>
       <c r="D25">
-        <v>5.39</v>
+        <v>4.32</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>350</v>
+        <v>450</v>
       </c>
       <c r="I25">
-        <v>2606</v>
+        <v>3391</v>
       </c>
       <c r="J25">
-        <v>18559</v>
+        <v>23147</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>47784.7</v>
+        <v>20305.6</v>
       </c>
       <c r="O25">
-        <v>47576</v>
+        <v>19276.4</v>
       </c>
       <c r="P25">
-        <v>48367.2</v>
+        <v>18838.7</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -5339,37 +5358,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>287.02</v>
+        <v>220.77</v>
       </c>
       <c r="C26">
-        <v>37.23</v>
+        <v>29.78</v>
       </c>
       <c r="D26">
-        <v>5.52</v>
+        <v>4.43</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>352</v>
+        <v>450</v>
       </c>
       <c r="I26">
-        <v>2678</v>
+        <v>3352</v>
       </c>
       <c r="J26">
-        <v>18088</v>
+        <v>22565</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>47162.1</v>
+        <v>20409.1</v>
       </c>
       <c r="O26">
-        <v>48922.2</v>
+        <v>19680.4</v>
       </c>
       <c r="P26">
-        <v>47488</v>
+        <v>19404.7</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -5377,37 +5396,37 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>149.69</v>
+        <v>110.16</v>
       </c>
       <c r="C27">
-        <v>19.28</v>
+        <v>16.64</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>2.71</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>674</v>
+        <v>908</v>
       </c>
       <c r="I27">
-        <v>5194</v>
+        <v>6006</v>
       </c>
       <c r="J27">
-        <v>33344</v>
+        <v>36850</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
-        <v>51259.5</v>
+        <v>20366.4</v>
       </c>
       <c r="O27">
-        <v>50236.4</v>
+        <v>19688.9</v>
       </c>
       <c r="P27">
-        <v>47698.1</v>
+        <v>19137.5</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -5415,37 +5434,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>68.39</v>
+        <v>60.18</v>
       </c>
       <c r="C28">
-        <v>13.81</v>
+        <v>11.99</v>
       </c>
       <c r="D28">
-        <v>2.47</v>
+        <v>2.22</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>1462</v>
+        <v>1666</v>
       </c>
       <c r="I28">
-        <v>7251</v>
+        <v>8349</v>
       </c>
       <c r="J28">
-        <v>40464</v>
+        <v>45116</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>45833.6</v>
+        <v>19779.8</v>
       </c>
       <c r="O28">
-        <v>49493.8</v>
+        <v>19229.6</v>
       </c>
       <c r="P28">
-        <v>48030.7</v>
+        <v>19341.9</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -5453,37 +5472,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>58.12</v>
+        <v>44.33</v>
       </c>
       <c r="C29">
-        <v>11.69</v>
+        <v>9.31</v>
       </c>
       <c r="D29">
-        <v>2.56</v>
+        <v>2.13</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>1717</v>
+        <v>2253</v>
       </c>
       <c r="I29">
-        <v>8562</v>
+        <v>10747</v>
       </c>
       <c r="J29">
-        <v>39103</v>
+        <v>46885</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>49364.1</v>
+        <v>19884.7</v>
       </c>
       <c r="O29">
-        <v>47890.3</v>
+        <v>18979</v>
       </c>
       <c r="P29">
-        <v>47521.4</v>
+        <v>19249.2</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -5491,37 +5510,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>46.72</v>
+        <v>34.38</v>
       </c>
       <c r="C30">
-        <v>11.23</v>
+        <v>8.32</v>
       </c>
       <c r="D30">
-        <v>2.52</v>
+        <v>2</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>2141</v>
+        <v>2913</v>
       </c>
       <c r="I30">
-        <v>8910</v>
+        <v>12030</v>
       </c>
       <c r="J30">
-        <v>39575</v>
+        <v>50025</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>47548.5</v>
+        <v>17244.1</v>
       </c>
       <c r="O30">
-        <v>47744.3</v>
+        <v>19476.6</v>
       </c>
       <c r="P30">
-        <v>47777.2</v>
+        <v>19198.1</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -5529,37 +5548,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>28.46</v>
+        <v>22.79</v>
       </c>
       <c r="C31">
-        <v>6.8</v>
+        <v>5.53</v>
       </c>
       <c r="D31">
-        <v>1.78</v>
+        <v>1.54</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>3506</v>
+        <v>4385</v>
       </c>
       <c r="I31">
-        <v>14724</v>
+        <v>18101</v>
       </c>
       <c r="J31">
-        <v>56181</v>
+        <v>64766</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>47755.7</v>
+        <v>19908.7</v>
       </c>
       <c r="O31">
-        <v>48732.4</v>
+        <v>19349.2</v>
       </c>
       <c r="P31">
-        <v>48094.5</v>
+        <v>19162.9</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -5567,37 +5586,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>26.98</v>
+        <v>21.21</v>
       </c>
       <c r="C32">
-        <v>6.63</v>
+        <v>5.4</v>
       </c>
       <c r="D32">
-        <v>1.66</v>
+        <v>1.48</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>3719</v>
+        <v>4717</v>
       </c>
       <c r="I32">
-        <v>15066</v>
+        <v>18524</v>
       </c>
       <c r="J32">
-        <v>60387</v>
+        <v>67421</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>47789.9</v>
+        <v>19389.3</v>
       </c>
       <c r="O32">
-        <v>47494.6</v>
+        <v>19033.9</v>
       </c>
       <c r="P32">
-        <v>47843.2</v>
+        <v>19122.4</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -5621,13 +5640,13 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="C39" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D39" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -5635,13 +5654,13 @@
         <v>43</v>
       </c>
       <c r="B40" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C40" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D40" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -5649,13 +5668,13 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C41" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D41" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -5663,13 +5682,848 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
+        <v>104</v>
+      </c>
+      <c r="C42" t="s">
+        <v>105</v>
+      </c>
+      <c r="D42" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>55</v>
+      </c>
+      <c r="B43" t="s">
+        <v>56</v>
+      </c>
+      <c r="C43" t="s">
+        <v>56</v>
+      </c>
+      <c r="D43" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P43"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>30.168</v>
+      </c>
+      <c r="C3">
+        <v>3.130506781332828E-05</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>54.284</v>
+      </c>
+      <c r="C4">
+        <v>4.938686577061096E-05</v>
+      </c>
+      <c r="F4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K4">
+        <v>1206</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>35.039</v>
+      </c>
+      <c r="C5">
+        <v>0.000180492827362639</v>
+      </c>
+      <c r="F5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" t="s">
+        <v>6</v>
+      </c>
+      <c r="K5">
+        <v>1976</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>33.485</v>
+      </c>
+      <c r="C6">
+        <v>0.0004194468537812072</v>
+      </c>
+      <c r="F6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K6">
+        <v>2209</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>19.648</v>
+      </c>
+      <c r="C7">
+        <v>0.001416775437222132</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7">
+        <v>4004</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>9.034000000000001</v>
+      </c>
+      <c r="C8">
+        <v>0.007310835927315079</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="J8" t="s">
+        <v>9</v>
+      </c>
+      <c r="K8">
+        <v>9442</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>8.281000000000001</v>
+      </c>
+      <c r="C9">
+        <v>0.01748041623111436</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" t="s">
+        <v>10</v>
+      </c>
+      <c r="K9">
+        <v>11135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10">
+        <v>6.74</v>
+      </c>
+      <c r="C10">
+        <v>0.04287579577376968</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="J10" t="s">
+        <v>11</v>
+      </c>
+      <c r="K10">
+        <v>14647</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>10.965</v>
+      </c>
+      <c r="C11">
+        <v>0.04474447006650164</v>
+      </c>
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="J11" t="s">
+        <v>12</v>
+      </c>
+      <c r="K11">
+        <v>9500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12">
+        <v>9.19</v>
+      </c>
+      <c r="C12">
+        <v>0.08487320527402402</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+      <c r="J12" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12">
+        <v>11866</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13">
+        <v>7.896</v>
+      </c>
+      <c r="C13">
+        <v>0.1794116187600719</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13">
+        <v>14643</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14">
+        <v>12.242</v>
+      </c>
+      <c r="C14">
+        <v>0.2273911526925453</v>
+      </c>
+      <c r="F14" t="s">
+        <v>15</v>
+      </c>
+      <c r="J14" t="s">
+        <v>15</v>
+      </c>
+      <c r="K14">
+        <v>10103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15">
+        <v>37.359</v>
+      </c>
+      <c r="C15">
+        <v>0.1298278517320922</v>
+      </c>
+      <c r="F15" t="s">
+        <v>16</v>
+      </c>
+      <c r="J15" t="s">
+        <v>16</v>
+      </c>
+      <c r="K15">
+        <v>3503</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16">
+        <v>58.936</v>
+      </c>
+      <c r="C16">
+        <v>0.1275543823075197</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>17</v>
+      </c>
+      <c r="K16">
+        <v>2319</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17">
+        <v>139.335</v>
+      </c>
+      <c r="C17">
+        <v>0.09498666906946536</v>
+      </c>
+      <c r="F17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K17">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18">
+        <v>15159.773</v>
+      </c>
+      <c r="C18">
+        <v>0.001319293056230302</v>
+      </c>
+      <c r="F18" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18" t="s">
+        <v>19</v>
+      </c>
+      <c r="K18">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G22" t="s">
+        <v>33</v>
+      </c>
+      <c r="M22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16">
+      <c r="B23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" t="s">
+        <v>32</v>
+      </c>
+      <c r="H23" t="s">
+        <v>30</v>
+      </c>
+      <c r="I23" t="s">
+        <v>31</v>
+      </c>
+      <c r="J23" t="s">
+        <v>32</v>
+      </c>
+      <c r="N23" t="s">
+        <v>30</v>
+      </c>
+      <c r="O23" t="s">
+        <v>31</v>
+      </c>
+      <c r="P23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16">
+      <c r="A24" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24">
+        <v>440.71</v>
+      </c>
+      <c r="C24">
+        <v>66.47</v>
+      </c>
+      <c r="D24">
+        <v>7.85</v>
+      </c>
+      <c r="G24" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24">
+        <v>226</v>
+      </c>
+      <c r="I24">
+        <v>1515</v>
+      </c>
+      <c r="J24">
+        <v>12734</v>
+      </c>
+      <c r="M24" t="s">
+        <v>21</v>
+      </c>
+      <c r="N24">
+        <v>53191.8</v>
+      </c>
+      <c r="O24">
+        <v>51155.3</v>
+      </c>
+      <c r="P24">
+        <v>47748.9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25">
+        <v>289.38</v>
+      </c>
+      <c r="C25">
+        <v>38.32</v>
+      </c>
+      <c r="D25">
+        <v>5.39</v>
+      </c>
+      <c r="G25" t="s">
+        <v>22</v>
+      </c>
+      <c r="H25">
+        <v>350</v>
+      </c>
+      <c r="I25">
+        <v>2606</v>
+      </c>
+      <c r="J25">
+        <v>18559</v>
+      </c>
+      <c r="M25" t="s">
+        <v>22</v>
+      </c>
+      <c r="N25">
+        <v>47784.7</v>
+      </c>
+      <c r="O25">
+        <v>47576</v>
+      </c>
+      <c r="P25">
+        <v>48367.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16">
+      <c r="A26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26">
+        <v>287.02</v>
+      </c>
+      <c r="C26">
+        <v>37.23</v>
+      </c>
+      <c r="D26">
+        <v>5.52</v>
+      </c>
+      <c r="G26" t="s">
+        <v>23</v>
+      </c>
+      <c r="H26">
+        <v>352</v>
+      </c>
+      <c r="I26">
+        <v>2678</v>
+      </c>
+      <c r="J26">
+        <v>18088</v>
+      </c>
+      <c r="M26" t="s">
+        <v>23</v>
+      </c>
+      <c r="N26">
+        <v>47162.1</v>
+      </c>
+      <c r="O26">
+        <v>48922.2</v>
+      </c>
+      <c r="P26">
+        <v>47488</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16">
+      <c r="A27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27">
+        <v>149.69</v>
+      </c>
+      <c r="C27">
+        <v>19.28</v>
+      </c>
+      <c r="D27">
+        <v>3</v>
+      </c>
+      <c r="G27" t="s">
+        <v>24</v>
+      </c>
+      <c r="H27">
+        <v>674</v>
+      </c>
+      <c r="I27">
+        <v>5194</v>
+      </c>
+      <c r="J27">
+        <v>33344</v>
+      </c>
+      <c r="M27" t="s">
+        <v>24</v>
+      </c>
+      <c r="N27">
+        <v>51259.5</v>
+      </c>
+      <c r="O27">
+        <v>50236.4</v>
+      </c>
+      <c r="P27">
+        <v>47698.1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16">
+      <c r="A28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28">
+        <v>68.39</v>
+      </c>
+      <c r="C28">
+        <v>13.81</v>
+      </c>
+      <c r="D28">
+        <v>2.47</v>
+      </c>
+      <c r="G28" t="s">
+        <v>25</v>
+      </c>
+      <c r="H28">
+        <v>1462</v>
+      </c>
+      <c r="I28">
+        <v>7251</v>
+      </c>
+      <c r="J28">
+        <v>40464</v>
+      </c>
+      <c r="M28" t="s">
+        <v>25</v>
+      </c>
+      <c r="N28">
+        <v>45833.6</v>
+      </c>
+      <c r="O28">
+        <v>49493.8</v>
+      </c>
+      <c r="P28">
+        <v>48030.7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16">
+      <c r="A29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29">
+        <v>58.12</v>
+      </c>
+      <c r="C29">
+        <v>11.69</v>
+      </c>
+      <c r="D29">
+        <v>2.56</v>
+      </c>
+      <c r="G29" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29">
+        <v>1717</v>
+      </c>
+      <c r="I29">
+        <v>8562</v>
+      </c>
+      <c r="J29">
+        <v>39103</v>
+      </c>
+      <c r="M29" t="s">
+        <v>26</v>
+      </c>
+      <c r="N29">
+        <v>49364.1</v>
+      </c>
+      <c r="O29">
+        <v>47890.3</v>
+      </c>
+      <c r="P29">
+        <v>47521.4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16">
+      <c r="A30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30">
+        <v>46.72</v>
+      </c>
+      <c r="C30">
+        <v>11.23</v>
+      </c>
+      <c r="D30">
+        <v>2.52</v>
+      </c>
+      <c r="G30" t="s">
+        <v>27</v>
+      </c>
+      <c r="H30">
+        <v>2141</v>
+      </c>
+      <c r="I30">
+        <v>8910</v>
+      </c>
+      <c r="J30">
+        <v>39575</v>
+      </c>
+      <c r="M30" t="s">
+        <v>27</v>
+      </c>
+      <c r="N30">
+        <v>47548.5</v>
+      </c>
+      <c r="O30">
+        <v>47744.3</v>
+      </c>
+      <c r="P30">
+        <v>47777.2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16">
+      <c r="A31" t="s">
+        <v>28</v>
+      </c>
+      <c r="B31">
+        <v>28.46</v>
+      </c>
+      <c r="C31">
+        <v>6.8</v>
+      </c>
+      <c r="D31">
+        <v>1.78</v>
+      </c>
+      <c r="G31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H31">
+        <v>3506</v>
+      </c>
+      <c r="I31">
+        <v>14724</v>
+      </c>
+      <c r="J31">
+        <v>56181</v>
+      </c>
+      <c r="M31" t="s">
+        <v>28</v>
+      </c>
+      <c r="N31">
+        <v>47755.7</v>
+      </c>
+      <c r="O31">
+        <v>48732.4</v>
+      </c>
+      <c r="P31">
+        <v>48094.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32">
+        <v>26.98</v>
+      </c>
+      <c r="C32">
+        <v>6.63</v>
+      </c>
+      <c r="D32">
+        <v>1.66</v>
+      </c>
+      <c r="G32" t="s">
+        <v>29</v>
+      </c>
+      <c r="H32">
+        <v>3719</v>
+      </c>
+      <c r="I32">
+        <v>15066</v>
+      </c>
+      <c r="J32">
+        <v>60387</v>
+      </c>
+      <c r="M32" t="s">
+        <v>29</v>
+      </c>
+      <c r="N32">
+        <v>47789.9</v>
+      </c>
+      <c r="O32">
+        <v>47494.6</v>
+      </c>
+      <c r="P32">
+        <v>47843.2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="B38" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" t="s">
+        <v>85</v>
+      </c>
+      <c r="C39" t="s">
+        <v>86</v>
+      </c>
+      <c r="D39" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" t="s">
         <v>108</v>
       </c>
+      <c r="C40" t="s">
+        <v>109</v>
+      </c>
+      <c r="D40" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" t="s">
+        <v>111</v>
+      </c>
+      <c r="C41" t="s">
+        <v>112</v>
+      </c>
+      <c r="D41" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" t="s">
+        <v>114</v>
+      </c>
       <c r="C42" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="D42" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="43" spans="1:4">

</xml_diff>

<commit_message>
Console closer to reels, readable win, calm spin button, coloured temple tiers in bonus, stage intro for Super/Divine Bonus, Jaguar King 250x all-or-nothing
</commit_message>
<xml_diff>
--- a/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
+++ b/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="120">
   <si>
     <t>Win Ranges</t>
   </si>
@@ -259,22 +259,31 @@
     <t>2385.1646356552055</t>
   </si>
   <si>
-    <t>2.0033775890958276</t>
-  </si>
-  <si>
-    <t>19217.340703473896</t>
-  </si>
-  <si>
-    <t>2.9797571339862867</t>
-  </si>
-  <si>
-    <t>19240.94819954831</t>
-  </si>
-  <si>
-    <t>6.051614714775488</t>
-  </si>
-  <si>
-    <t>19064.456788819545</t>
+    <t>2.3556115501687813</t>
+  </si>
+  <si>
+    <t>42428</t>
+  </si>
+  <si>
+    <t>24490.871565129466</t>
+  </si>
+  <si>
+    <t>2.898995916771497</t>
+  </si>
+  <si>
+    <t>34499</t>
+  </si>
+  <si>
+    <t>23669.497949069744</t>
+  </si>
+  <si>
+    <t>4.337740457192749</t>
+  </si>
+  <si>
+    <t>23073</t>
+  </si>
+  <si>
+    <t>23590.6117441935</t>
   </si>
   <si>
     <t>1.0</t>
@@ -3231,8 +3240,8 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>69</v>
+      <c r="B2">
+        <v>2.5</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -3244,7 +3253,7 @@
         <v>3</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -3352,10 +3361,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>5.693</v>
+        <v>24.528</v>
       </c>
       <c r="C8">
-        <v>0.03023891102145014</v>
+        <v>0.005810272764231779</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -3364,7 +3373,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>17403</v>
+        <v>5985</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -3372,10 +3381,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>3.862</v>
+        <v>11.101</v>
       </c>
       <c r="C9">
-        <v>0.09066130701457091</v>
+        <v>0.02576976595560151</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -3384,7 +3393,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>25791</v>
+        <v>11321</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -3392,10 +3401,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>3.542</v>
+        <v>6.836</v>
       </c>
       <c r="C10">
-        <v>0.1922369331082189</v>
+        <v>0.08188315694622177</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -3404,7 +3413,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>28256</v>
+        <v>15874</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -3412,10 +3421,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>8.654</v>
+        <v>11.154</v>
       </c>
       <c r="C11">
-        <v>0.1354056206207358</v>
+        <v>0.08504438462745631</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -3424,7 +3433,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>11613</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -3432,10 +3441,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>10.222</v>
+        <v>9.909000000000001</v>
       </c>
       <c r="C12">
-        <v>0.1816094882657492</v>
+        <v>0.1531399797108261</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -3444,7 +3453,7 @@
         <v>13</v>
       </c>
       <c r="K12">
-        <v>9865</v>
+        <v>8766</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -3452,10 +3461,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>19.619</v>
+        <v>12.23</v>
       </c>
       <c r="C13">
-        <v>0.1704128380538051</v>
+        <v>0.2226834962187363</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -3464,7 +3473,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>5162</v>
+        <v>6250</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -3472,10 +3481,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>68.173</v>
+        <v>27.502</v>
       </c>
       <c r="C14">
-        <v>0.09616335272235986</v>
+        <v>0.1961564016657589</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -3484,7 +3493,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>1493</v>
+        <v>2388</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -3492,10 +3501,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>407.256</v>
+        <v>129.67</v>
       </c>
       <c r="C15">
-        <v>0.02835934303822878</v>
+        <v>0.07330376986540889</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -3504,7 +3513,7 @@
         <v>16</v>
       </c>
       <c r="K15">
-        <v>251</v>
+        <v>445</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -3512,10 +3521,10 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>801.259</v>
+        <v>211.727</v>
       </c>
       <c r="C16">
-        <v>0.02267627180529015</v>
+        <v>0.06894440260236637</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
@@ -3524,7 +3533,7 @@
         <v>17</v>
       </c>
       <c r="K16">
-        <v>128</v>
+        <v>248</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -3532,10 +3541,10 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>2861.043</v>
+        <v>598.707</v>
       </c>
       <c r="C17">
-        <v>0.01126830047061499</v>
+        <v>0.0443398893724935</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -3544,7 +3553,7 @@
         <v>18</v>
       </c>
       <c r="K17">
-        <v>36</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -3552,10 +3561,10 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>51672.431</v>
+        <v>13677.645</v>
       </c>
       <c r="C18">
-        <v>0.000967633970204461</v>
+        <v>0.002924480015698779</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
@@ -3564,7 +3573,7 @@
         <v>19</v>
       </c>
       <c r="K18">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -3612,37 +3621,37 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>33259.08</v>
+        <v>0</v>
       </c>
       <c r="C24">
-        <v>951.84</v>
+        <v>1373.14</v>
       </c>
       <c r="D24">
-        <v>66.81999999999999</v>
+        <v>112.16</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I24">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="J24">
-        <v>1496</v>
+        <v>897</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>9324.6</v>
+        <v>0</v>
       </c>
       <c r="O24">
-        <v>16862.1</v>
+        <v>16831.4</v>
       </c>
       <c r="P24">
-        <v>18667.8</v>
+        <v>24557.2</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -3650,37 +3659,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>6645.09</v>
+        <v>9648.08</v>
       </c>
       <c r="C25">
-        <v>454.9</v>
+        <v>889.61</v>
       </c>
       <c r="D25">
-        <v>38.14</v>
+        <v>63.19</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I25">
-        <v>220</v>
+        <v>112</v>
       </c>
       <c r="J25">
-        <v>2622</v>
+        <v>1574</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>10299.3</v>
+        <v>27246.2</v>
       </c>
       <c r="O25">
-        <v>21426</v>
+        <v>31158.6</v>
       </c>
       <c r="P25">
-        <v>18274.9</v>
+        <v>24230.6</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -3688,37 +3697,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>2130.69</v>
+        <v>3326.28</v>
       </c>
       <c r="C26">
-        <v>246.88</v>
+        <v>427.77</v>
       </c>
       <c r="D26">
-        <v>21.79</v>
+        <v>36.35</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="I26">
-        <v>405</v>
+        <v>235</v>
       </c>
       <c r="J26">
-        <v>4590</v>
+        <v>2756</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>20614.8</v>
+        <v>32309.7</v>
       </c>
       <c r="O26">
-        <v>18041.2</v>
+        <v>21371.2</v>
       </c>
       <c r="P26">
-        <v>20074.7</v>
+        <v>23757.9</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -3726,37 +3735,37 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>1351.57</v>
+        <v>2945.71</v>
       </c>
       <c r="C27">
-        <v>154.87</v>
+        <v>282.13</v>
       </c>
       <c r="D27">
-        <v>15.42</v>
+        <v>26.17</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="I27">
-        <v>646</v>
+        <v>352</v>
       </c>
       <c r="J27">
-        <v>6484</v>
+        <v>3847</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
-        <v>20884.4</v>
+        <v>18675</v>
       </c>
       <c r="O27">
-        <v>20882.1</v>
+        <v>25497.6</v>
       </c>
       <c r="P27">
-        <v>19187.5</v>
+        <v>23146.8</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -3764,37 +3773,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>469.08</v>
+        <v>897.83</v>
       </c>
       <c r="C28">
-        <v>66.93000000000001</v>
+        <v>109.98</v>
       </c>
       <c r="D28">
-        <v>8.9</v>
+        <v>15.13</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>213</v>
+        <v>114</v>
       </c>
       <c r="I28">
-        <v>1494</v>
+        <v>915</v>
       </c>
       <c r="J28">
-        <v>11234</v>
+        <v>6629</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>16892</v>
+        <v>23333.8</v>
       </c>
       <c r="O28">
-        <v>19703.3</v>
+        <v>25939.6</v>
       </c>
       <c r="P28">
-        <v>19696.9</v>
+        <v>23661.6</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -3802,37 +3811,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>303.83</v>
+        <v>555.8</v>
       </c>
       <c r="C29">
-        <v>44.39</v>
+        <v>75.54000000000001</v>
       </c>
       <c r="D29">
-        <v>6.52</v>
+        <v>10.8</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>329</v>
+        <v>180</v>
       </c>
       <c r="I29">
-        <v>2253</v>
+        <v>1319</v>
       </c>
       <c r="J29">
-        <v>15337</v>
+        <v>9233</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>17688.7</v>
+        <v>32903.9</v>
       </c>
       <c r="O29">
-        <v>18841.8</v>
+        <v>25272.6</v>
       </c>
       <c r="P29">
-        <v>19372.9</v>
+        <v>25103.5</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -3840,37 +3849,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>238.04</v>
+        <v>406.6</v>
       </c>
       <c r="C30">
-        <v>37.31</v>
+        <v>64.13</v>
       </c>
       <c r="D30">
-        <v>5.21</v>
+        <v>8.51</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>420</v>
+        <v>244</v>
       </c>
       <c r="I30">
-        <v>2681</v>
+        <v>1551</v>
       </c>
       <c r="J30">
-        <v>19189</v>
+        <v>11768</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>17797.5</v>
+        <v>22938.5</v>
       </c>
       <c r="O30">
-        <v>20006.3</v>
+        <v>28286.1</v>
       </c>
       <c r="P30">
-        <v>19265.2</v>
+        <v>22817.8</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -3878,37 +3887,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>178.19</v>
+        <v>308.99</v>
       </c>
       <c r="C31">
-        <v>34.81</v>
+        <v>58.16</v>
       </c>
       <c r="D31">
-        <v>5.79</v>
+        <v>9.59</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>561</v>
+        <v>323</v>
       </c>
       <c r="I31">
-        <v>2873</v>
+        <v>1713</v>
       </c>
       <c r="J31">
-        <v>17259</v>
+        <v>10446</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>16830</v>
+        <v>22221.1</v>
       </c>
       <c r="O31">
-        <v>19290.5</v>
+        <v>25055.7</v>
       </c>
       <c r="P31">
-        <v>18845.6</v>
+        <v>23510.1</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -3916,37 +3925,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>216.84</v>
+        <v>383.31</v>
       </c>
       <c r="C32">
-        <v>38.55</v>
+        <v>65.3</v>
       </c>
       <c r="D32">
-        <v>5.95</v>
+        <v>9.85</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>461</v>
+        <v>265</v>
       </c>
       <c r="I32">
-        <v>2594</v>
+        <v>1525</v>
       </c>
       <c r="J32">
-        <v>16819</v>
+        <v>10161</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>17889.5</v>
+        <v>18142.7</v>
       </c>
       <c r="O32">
-        <v>18550.2</v>
+        <v>23406.9</v>
       </c>
       <c r="P32">
-        <v>19039.8</v>
+        <v>23173.3</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -4001,10 +4010,10 @@
         <v>79</v>
       </c>
       <c r="C41" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="D41" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -4012,13 +4021,13 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C42" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="D42" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -4026,13 +4035,13 @@
         <v>55</v>
       </c>
       <c r="B43" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C43" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="D43" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -4805,13 +4814,13 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C39" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D39" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -4819,13 +4828,13 @@
         <v>43</v>
       </c>
       <c r="B40" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D40" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -4833,13 +4842,13 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C41" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D41" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -4847,13 +4856,13 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C42" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D42" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -5640,13 +5649,13 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C39" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D39" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -5654,13 +5663,13 @@
         <v>43</v>
       </c>
       <c r="B40" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C40" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D40" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -5668,13 +5677,13 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C41" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D41" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -5682,13 +5691,13 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C42" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D42" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -6475,13 +6484,13 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C39" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D39" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -6489,13 +6498,13 @@
         <v>43</v>
       </c>
       <c r="B40" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C40" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D40" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -6503,13 +6512,13 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C41" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D41" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -6517,13 +6526,13 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C42" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D42" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="43" spans="1:4">

</xml_diff>

<commit_message>
Smaller spin button, no blue dots, distinct temple tiers, big-win animation in Jaguar spins from 20x bet, Jaguar Spin can miss, clearer feature texts
</commit_message>
<xml_diff>
--- a/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
+++ b/math/temple_of_ascent/library/temple_of_ascent_full_statistics.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="120">
   <si>
     <t>Win Ranges</t>
   </si>
@@ -232,31 +232,31 @@
     <t>NaN</t>
   </si>
   <si>
-    <t>2.003350238093352</t>
-  </si>
-  <si>
-    <t>49916</t>
-  </si>
-  <si>
-    <t>2397.7635207342105</t>
-  </si>
-  <si>
-    <t>2.979494306817953</t>
-  </si>
-  <si>
-    <t>33561</t>
-  </si>
-  <si>
-    <t>2410.6287570062077</t>
-  </si>
-  <si>
-    <t>6.052948730902352</t>
-  </si>
-  <si>
-    <t>16523</t>
-  </si>
-  <si>
-    <t>2385.1646356552055</t>
+    <t>2.0831917056990923</t>
+  </si>
+  <si>
+    <t>48060</t>
+  </si>
+  <si>
+    <t>2365.9187649319065</t>
+  </si>
+  <si>
+    <t>2.934000932128004</t>
+  </si>
+  <si>
+    <t>34052</t>
+  </si>
+  <si>
+    <t>2414.637904079269</t>
+  </si>
+  <si>
+    <t>5.582355642339494</t>
+  </si>
+  <si>
+    <t>17888</t>
+  </si>
+  <si>
+    <t>2463.477237919986</t>
   </si>
   <si>
     <t>2.3556115501687813</t>
@@ -2405,8 +2405,8 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>69</v>
+      <c r="B2">
+        <v>4</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -2418,7 +2418,7 @@
         <v>3</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -2466,10 +2466,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>10.295</v>
+        <v>20.782</v>
       </c>
       <c r="C5">
-        <v>0.0138903201420959</v>
+        <v>0.006970980364059028</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -2478,7 +2478,7 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>9817</v>
+        <v>6815</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -2486,10 +2486,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>4.284</v>
+        <v>7.289</v>
       </c>
       <c r="C6">
-        <v>0.0664254236666955</v>
+        <v>0.03935342602107955</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -2498,7 +2498,7 @@
         <v>7</v>
       </c>
       <c r="K6">
-        <v>23475</v>
+        <v>16370</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -2506,10 +2506,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>3.363</v>
+        <v>4.746</v>
       </c>
       <c r="C7">
-        <v>0.1646879761909692</v>
+        <v>0.1178561042819559</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -2518,7 +2518,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>29742</v>
+        <v>20998</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -2526,10 +2526,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>3.697</v>
+        <v>4.264</v>
       </c>
       <c r="C8">
-        <v>0.3254238811364674</v>
+        <v>0.2881848707489899</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -2538,7 +2538,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>26886</v>
+        <v>18797</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -2546,10 +2546,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>13.602</v>
+        <v>12.555</v>
       </c>
       <c r="C9">
-        <v>0.1979259633080359</v>
+        <v>0.2171242798065412</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -2558,7 +2558,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>7257</v>
+        <v>5026</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -2566,10 +2566,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>45.558</v>
+        <v>33.69</v>
       </c>
       <c r="C10">
-        <v>0.1164848064240701</v>
+        <v>0.159524199188527</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -2578,7 +2578,7 @@
         <v>11</v>
       </c>
       <c r="K10">
-        <v>2154</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -2586,10 +2586,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>241.074</v>
+        <v>158.384</v>
       </c>
       <c r="C11">
-        <v>0.03892073825577238</v>
+        <v>0.05909521424552657</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
@@ -2598,7 +2598,7 @@
         <v>12</v>
       </c>
       <c r="K11">
-        <v>405</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2606,10 +2606,10 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>645.24</v>
+        <v>364.071</v>
       </c>
       <c r="C12">
-        <v>0.02241878989383664</v>
+        <v>0.04002940780295863</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -2618,7 +2618,7 @@
         <v>13</v>
       </c>
       <c r="K12">
-        <v>201</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -2626,10 +2626,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>2389.354</v>
+        <v>1064.166</v>
       </c>
       <c r="C13">
-        <v>0.01102882559985251</v>
+        <v>0.02528468130669921</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
@@ -2638,7 +2638,7 @@
         <v>14</v>
       </c>
       <c r="K13">
-        <v>54</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2646,10 +2646,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>16779.173</v>
+        <v>7055.807</v>
       </c>
       <c r="C14">
-        <v>0.002793275777131588</v>
+        <v>0.006576837355965956</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -2658,7 +2658,7 @@
         <v>15</v>
       </c>
       <c r="K14">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -2786,37 +2786,37 @@
         <v>21</v>
       </c>
       <c r="B24">
-        <v>33426.12</v>
+        <v>115309.78</v>
       </c>
       <c r="C24">
-        <v>952.36</v>
+        <v>1184.34</v>
       </c>
       <c r="D24">
-        <v>66.87</v>
+        <v>95.98</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I24">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="J24">
-        <v>1496</v>
+        <v>1044</v>
       </c>
       <c r="M24" t="s">
         <v>21</v>
       </c>
       <c r="N24">
-        <v>1033.8</v>
+        <v>800</v>
       </c>
       <c r="O24">
-        <v>2192.4</v>
+        <v>2639.3</v>
       </c>
       <c r="P24">
-        <v>2319.5</v>
+        <v>2488</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -2824,37 +2824,37 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>6686.53</v>
+        <v>10201.17</v>
       </c>
       <c r="C25">
-        <v>454.43</v>
+        <v>618.16</v>
       </c>
       <c r="D25">
-        <v>38.12</v>
+        <v>54.18</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
       </c>
       <c r="H25">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I25">
-        <v>220</v>
+        <v>153</v>
       </c>
       <c r="J25">
-        <v>2622</v>
+        <v>1837</v>
       </c>
       <c r="M25" t="s">
         <v>22</v>
       </c>
       <c r="N25">
-        <v>1276.3</v>
+        <v>779.1</v>
       </c>
       <c r="O25">
-        <v>2638</v>
+        <v>2995.5</v>
       </c>
       <c r="P25">
-        <v>2297.4</v>
+        <v>2265.6</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -2862,37 +2862,37 @@
         <v>23</v>
       </c>
       <c r="B26">
-        <v>2123.26</v>
+        <v>2939.64</v>
       </c>
       <c r="C26">
-        <v>246.76</v>
+        <v>366.45</v>
       </c>
       <c r="D26">
-        <v>21.79</v>
+        <v>30.69</v>
       </c>
       <c r="G26" t="s">
         <v>23</v>
       </c>
       <c r="H26">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="I26">
-        <v>405</v>
+        <v>274</v>
       </c>
       <c r="J26">
-        <v>4590</v>
+        <v>3234</v>
       </c>
       <c r="M26" t="s">
         <v>23</v>
       </c>
       <c r="N26">
-        <v>2582.2</v>
+        <v>2450.4</v>
       </c>
       <c r="O26">
-        <v>2331.5</v>
+        <v>2287.8</v>
       </c>
       <c r="P26">
-        <v>2493.4</v>
+        <v>2675.4</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -2900,37 +2900,37 @@
         <v>24</v>
       </c>
       <c r="B27">
-        <v>1355.19</v>
+        <v>1976.93</v>
       </c>
       <c r="C27">
-        <v>154.76</v>
+        <v>225.68</v>
       </c>
       <c r="D27">
-        <v>15.42</v>
+        <v>22.18</v>
       </c>
       <c r="G27" t="s">
         <v>24</v>
       </c>
       <c r="H27">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="I27">
-        <v>646</v>
+        <v>438</v>
       </c>
       <c r="J27">
-        <v>6484</v>
+        <v>4523</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
       </c>
       <c r="N27">
-        <v>2647.5</v>
+        <v>3046.5</v>
       </c>
       <c r="O27">
-        <v>2630.3</v>
+        <v>2970.8</v>
       </c>
       <c r="P27">
-        <v>2418.5</v>
+        <v>2346.6</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -2938,37 +2938,37 @@
         <v>25</v>
       </c>
       <c r="B28">
-        <v>470.71</v>
+        <v>737.9400000000001</v>
       </c>
       <c r="C28">
-        <v>66.95</v>
+        <v>95.12</v>
       </c>
       <c r="D28">
-        <v>8.9</v>
+        <v>12.79</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28">
-        <v>213</v>
+        <v>137</v>
       </c>
       <c r="I28">
-        <v>1494</v>
+        <v>1069</v>
       </c>
       <c r="J28">
-        <v>11234</v>
+        <v>7848</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
       </c>
       <c r="N28">
-        <v>2194.7</v>
+        <v>2730.6</v>
       </c>
       <c r="O28">
-        <v>2444.1</v>
+        <v>2179.2</v>
       </c>
       <c r="P28">
-        <v>2450.3</v>
+        <v>2389.8</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -2976,37 +2976,37 @@
         <v>26</v>
       </c>
       <c r="B29">
-        <v>303.86</v>
+        <v>446.82</v>
       </c>
       <c r="C29">
-        <v>44.37</v>
+        <v>63.98</v>
       </c>
       <c r="D29">
-        <v>6.52</v>
+        <v>9.33</v>
       </c>
       <c r="G29" t="s">
         <v>26</v>
       </c>
       <c r="H29">
-        <v>329</v>
+        <v>226</v>
       </c>
       <c r="I29">
-        <v>2253</v>
+        <v>1566</v>
       </c>
       <c r="J29">
-        <v>15337</v>
+        <v>10718</v>
       </c>
       <c r="M29" t="s">
         <v>26</v>
       </c>
       <c r="N29">
-        <v>2273.8</v>
+        <v>2279.6</v>
       </c>
       <c r="O29">
-        <v>2375.8</v>
+        <v>2257.2</v>
       </c>
       <c r="P29">
-        <v>2415.3</v>
+        <v>2457.4</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -3014,37 +3014,37 @@
         <v>27</v>
       </c>
       <c r="B30">
-        <v>238.13</v>
+        <v>333.25</v>
       </c>
       <c r="C30">
-        <v>37.29</v>
+        <v>53.71</v>
       </c>
       <c r="D30">
-        <v>5.21</v>
+        <v>7.37</v>
       </c>
       <c r="G30" t="s">
         <v>27</v>
       </c>
       <c r="H30">
-        <v>420</v>
+        <v>305</v>
       </c>
       <c r="I30">
-        <v>2681</v>
+        <v>1862</v>
       </c>
       <c r="J30">
-        <v>19189</v>
+        <v>13526</v>
       </c>
       <c r="M30" t="s">
         <v>27</v>
       </c>
       <c r="N30">
-        <v>2232.6</v>
+        <v>1804.8</v>
       </c>
       <c r="O30">
-        <v>2487.7</v>
+        <v>2534.9</v>
       </c>
       <c r="P30">
-        <v>2411.6</v>
+        <v>2439.8</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -3052,37 +3052,37 @@
         <v>28</v>
       </c>
       <c r="B31">
-        <v>178.2</v>
+        <v>259.09</v>
       </c>
       <c r="C31">
-        <v>34.8</v>
+        <v>50.02</v>
       </c>
       <c r="D31">
-        <v>5.79</v>
+        <v>8.25</v>
       </c>
       <c r="G31" t="s">
         <v>28</v>
       </c>
       <c r="H31">
-        <v>561</v>
+        <v>392</v>
       </c>
       <c r="I31">
-        <v>2873</v>
+        <v>1984</v>
       </c>
       <c r="J31">
-        <v>17259</v>
+        <v>12139</v>
       </c>
       <c r="M31" t="s">
         <v>28</v>
       </c>
       <c r="N31">
-        <v>2161.5</v>
+        <v>1879.2</v>
       </c>
       <c r="O31">
-        <v>2424</v>
+        <v>2441.4</v>
       </c>
       <c r="P31">
-        <v>2360.5</v>
+        <v>2388.2</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -3090,37 +3090,37 @@
         <v>29</v>
       </c>
       <c r="B32">
-        <v>217.05</v>
+        <v>325.31</v>
       </c>
       <c r="C32">
-        <v>38.54</v>
+        <v>55.54</v>
       </c>
       <c r="D32">
-        <v>5.95</v>
+        <v>8.51</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
       </c>
       <c r="H32">
-        <v>461</v>
+        <v>314</v>
       </c>
       <c r="I32">
-        <v>2594</v>
+        <v>1795</v>
       </c>
       <c r="J32">
-        <v>16819</v>
+        <v>11761</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
       </c>
       <c r="N32">
-        <v>2280.3</v>
+        <v>2229.7</v>
       </c>
       <c r="O32">
-        <v>2322.5</v>
+        <v>2313.8</v>
       </c>
       <c r="P32">
-        <v>2377.3</v>
+        <v>2360.2</v>
       </c>
     </row>
     <row r="37" spans="1:4">

</xml_diff>